<commit_message>
Committing Generated Files 44
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with correct URL and UI elements</t>
+          <t>Verify login page loads and all required UI elements are visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open a browser
-Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the page URL and login form elements</t>
+          <t>Navigate to http://172.21.166.115/washtabui/login?data=undefined
+Observe the login page
+Verify username_textbox, password_textbox, sign_in_button, home_navigation_button and back_navigation_button are displayed</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Browser URL remains http://172.21.166.115/washtabui/login?data=undefined and username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible on the page</t>
+          <t>Login page loads successfully and username_textbox, password_textbox, SIGN IN button, home_navigation_button and back_navigation_button are visible and enabled for user interaction</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify username textbox is visible and accepts input</t>
+          <t>Verify successful login with valid username and password</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Locate the username textbox
-Click inside the username textbox and type a sample username</t>
+          <t>Navigate to the login page
+Enter hacklarr in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Username textbox is visible, enabled, receives focus when clicked, and displays the entered text</t>
+          <t>User authentication succeeds and application redirects to home page with URL http://172.21.166.115/washtabui/home and login page is no longer displayed</t>
         </is>
       </c>
     </row>
@@ -540,12 +541,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password textbox is visible and masks characters</t>
+          <t>Verify login fails with invalid username and valid password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -556,14 +557,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Locate the password textbox
-Type a sample password into the password textbox</t>
+          <t>Navigate to the login page
+Enter invalidUser in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Password textbox is visible and enabled and the entered characters are masked (shown as dots or asterisks) instead of plain text</t>
+          <t>Authentication is rejected, an error or sign-in failure message is displayed, and the browser remains on the login page without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -575,12 +577,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify SIGN IN button is visible and clickable</t>
+          <t>Verify login fails with valid username and incorrect password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -591,14 +593,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Locate the SIGN IN button
-Click the SIGN IN button without entering credentials</t>
+          <t>Navigate to the login page
+Enter hacklarr in username_textbox
+Enter WrongPassword123 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SIGN IN button is visible and clickable and the login form remains on the login page indicating login cannot proceed without valid credentials</t>
+          <t>Authentication fails, a visible login error message is displayed, and the application remains on the login page without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -610,12 +613,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify successful login with valid credentials</t>
+          <t>Verify login fails when both username and password are invalid</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -626,15 +629,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter invalidUser in username_textbox
+Enter invalidPassword in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and redirected to the home page where the browser URL becomes http://172.21.166.115/washtabui/home and the home page UI is displayed</t>
+          <t>Login attempt is rejected, a visible authentication failure message appears, and the page remains on the login URL without navigation to the home page</t>
         </is>
       </c>
     </row>
@@ -646,7 +649,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify login fails with incorrect password</t>
+          <t>Verify validation when username field is empty</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -662,15 +665,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter hacklarr in the username textbox
-Enter incorrectPassword in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Leave username_textbox empty
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, user remains on the login page URL, the application does not navigate to the home page, and a visible authentication failure or sign‑in error message is displayed</t>
+          <t>Login submission is blocked, a validation or error indication appears for username_textbox, and the login page remains displayed without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -682,7 +685,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login fails with invalid username</t>
+          <t>Verify validation when password field is empty</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -698,15 +701,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter invaliduser in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter hacklarr in username_textbox
+Leave password_textbox empty
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication fails and the application remains on the login page without redirecting to the home page and an authentication failure indication is visible</t>
+          <t>Login submission is prevented, a validation or error indication appears for password_textbox, and the user remains on the login page</t>
         </is>
       </c>
     </row>
@@ -718,7 +721,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login fails with both username and password invalid</t>
+          <t>Verify validation when both username and password fields are empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -734,15 +737,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter invaliduser in the username textbox
-Enter invalidPassword in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Leave username_textbox empty
+Leave password_textbox empty
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication is rejected, the login page remains displayed, and no navigation to http://172.21.166.115/washtabui/home occurs</t>
+          <t>Submission is rejected, validation messages or visual error indicators appear for both fields, and the login page remains displayed without navigation</t>
         </is>
       </c>
     </row>
@@ -754,12 +757,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify login attempt with empty username and password</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -770,15 +773,13 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Leave the username textbox empty
-Leave the password textbox empty
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter text into password_textbox</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Login is rejected and the user remains on the login page without navigation to the home page</t>
+          <t>Characters typed into password_textbox appear masked as dots or bullet characters and the actual text value is not visible on the screen</t>
         </is>
       </c>
     </row>
@@ -790,12 +791,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify login attempt with username only</t>
+          <t>Verify home navigation button redirects user to home page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -806,15 +807,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter hacklarr in the username textbox
-Leave the password textbox empty
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Click home_navigation_button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Authentication does not succeed and the application stays on the login page without redirecting to the home page</t>
+          <t>Application navigates to the home page and the browser URL changes to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -826,12 +825,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify login attempt with password only</t>
+          <t>Verify back navigation button redirects user to home page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -842,15 +841,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Leave the username textbox empty
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Click back_navigation_button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Authentication does not succeed and the login page remains displayed without redirecting to the home page</t>
+          <t>Application navigates away from the login page and loads the home page with URL http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -862,12 +859,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify navigation using home navigation button</t>
+          <t>Verify login behavior when username contains leading and trailing spaces</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -878,13 +875,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Click the home navigation button</t>
+          <t>Navigate to the login page
+Enter space hacklarr space in username_textbox
+Enter Icstunnel1 in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home</t>
+          <t>System either trims the whitespace and authenticates the user successfully redirecting to http://172.21.166.115/washtabui/home, or rejects the login attempt with a visible error while remaining on the login page</t>
         </is>
       </c>
     </row>
@@ -896,12 +895,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify navigation using back navigation button</t>
+          <t>Verify login attempt using whitespace-only values</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -912,13 +911,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Click the back navigation button</t>
+          <t>Navigate to the login page
+Enter only spaces in username_textbox
+Enter only spaces in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Application navigates to the home page and the browser URL becomes http://172.21.166.115/washtabui/home</t>
+          <t>System rejects the login attempt, displays a validation or authentication error message, and remains on the login page without redirecting to the home page</t>
         </is>
       </c>
     </row>
@@ -930,7 +931,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify login with leading and trailing whitespace in username</t>
+          <t>Verify system behavior when SIGN IN button is clicked multiple times rapidly</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -946,15 +947,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter ' hacklarr ' including leading and trailing spaces in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter hacklarr in username_textbox
+Enter Icstunnel1 in password_textbox
+Rapidly click sign_in_button multiple times</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Application processes the input without UI errors; user is either authenticated and redirected to the home page if whitespace is trimmed or login fails and the login page remains displayed</t>
+          <t>Application processes the authentication request only once and redirects to the home page a single time without duplicate requests, page errors, or unexpected behavior</t>
         </is>
       </c>
     </row>
@@ -966,7 +967,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login with very long username input</t>
+          <t>Verify login attempt with very long username and password values</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -982,15 +983,15 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter a very long string exceeding typical username length in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
+          <t>Navigate to the login page
+Enter a very long string exceeding typical username length in username_textbox
+Enter a very long string exceeding typical password length in password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Application handles the long input without crashing or breaking the UI and authentication fails while remaining on the login page</t>
+          <t>Application safely rejects the authentication attempt and remains on the login page without UI breakage, application crash, or unexpected navigation</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1003,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify repeated clicking of SIGN IN button during login attempt</t>
+          <t>Verify login submission using Enter key from password field</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1018,15 +1019,15 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
-Rapidly click the SIGN IN button multiple times</t>
+          <t>Navigate to the login page
+Enter hacklarr in username_textbox
+Enter Icstunnel1 in password_textbox
+Press Enter key while cursor focus is inside password_textbox</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Application processes the login request once and redirects to the home page a single time without duplicate redirects or UI errors</t>
+          <t>Pressing Enter triggers the login action and the user is successfully authenticated and redirected to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1039,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login submission using Enter key</t>
+          <t>Verify login using copy and paste for credentials</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1054,87 +1055,15 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Enter hacklarr in the username textbox
-Enter Icstunnel1 in the password textbox
-Press the Enter key while focused on the password textbox</t>
+          <t>Navigate to the login page
+Copy the value hacklarr and paste it into username_textbox
+Copy the value Icstunnel1 and paste it into password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Login form submits and the user is redirected to the home page with URL http://172.21.166.115/washtabui/home</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify login using pasted credentials</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Paste hacklarr into the username textbox
-Paste Icstunnel1 into the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Application accepts pasted values and authenticates successfully and redirects to http://172.21.166.115/washtabui/home</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WT-LOGIN19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Verify username case sensitivity during login</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Open the login page URL
-Enter HACKLARR in the username textbox
-Enter Icstunnel1 in the password textbox
-Click the SIGN IN button</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>If the system enforces case sensitivity login fails and the user remains on the login page with an authentication error; otherwise the user is redirected to the home page</t>
+          <t>Pasted credentials are accepted as valid input and user authentication succeeds with redirection to http://172.21.166.115/washtabui/home</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 45
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads and all required UI elements are visible</t>
+          <t>Verify login page loads with all required UI elements</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,13 +487,12 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page
-Verify username_textbox, password_textbox, sign_in_button, home_navigation_button and back_navigation_button are displayed</t>
+Observe the login page UI</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads successfully and username_textbox, password_textbox, SIGN IN button, home_navigation_button and back_navigation_button are visible and enabled for user interaction</t>
+          <t>Login page loads at the specified URL and username_textbox, password_textbox, sign_in_button, home_navigation_button, and back_navigation_button are visible, enabled, and ready for user interaction.</t>
         </is>
       </c>
     </row>
@@ -505,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login with valid username and password</t>
+          <t>Verify successful login with valid credentials</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,14 +521,14 @@
       <c r="F3" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in username_textbox
-Enter Icstunnel1 in password_textbox
+Enter hacklarr into username_textbox
+Enter Icstunnel1 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User authentication succeeds and application redirects to home page with URL http://172.21.166.115/washtabui/home and login page is no longer displayed</t>
+          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home where the home page UI is visible and the login page is no longer displayed.</t>
         </is>
       </c>
     </row>
@@ -541,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify login fails with invalid username and valid password</t>
+          <t>Verify login fails with valid username and invalid password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,14 +557,14 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter invalidUser in username_textbox
-Enter Icstunnel1 in password_textbox
+Enter hacklarr into username_textbox
+Enter WrongPassword123 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Authentication is rejected, an error or sign-in failure message is displayed, and the browser remains on the login page without redirecting to the home page</t>
+          <t>Authentication is rejected, the user remains on the login page URL, and a visible error message indicating invalid or incorrect credentials is displayed.</t>
         </is>
       </c>
     </row>
@@ -577,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with valid username and incorrect password</t>
+          <t>Verify login fails with invalid username and valid password</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -594,14 +593,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in username_textbox
-Enter WrongPassword123 in password_textbox
+Enter invaliduser into username_textbox
+Enter Icstunnel1 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails, a visible login error message is displayed, and the application remains on the login page without redirecting to the home page</t>
+          <t>Authentication fails, the application stays on the login page URL, and a visible message indicating invalid or incorrect credentials is displayed.</t>
         </is>
       </c>
     </row>
@@ -613,7 +612,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails when both username and password are invalid</t>
+          <t>Verify login fails when both username and password are incorrect</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -630,14 +629,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter invalidUser in username_textbox
-Enter invalidPassword in password_textbox
+Enter wronguser into username_textbox
+Enter wrongpass into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Login attempt is rejected, a visible authentication failure message appears, and the page remains on the login URL without navigation to the home page</t>
+          <t>Authentication fails, the application remains on the login page, and a visible invalid credentials error message is shown.</t>
         </is>
       </c>
     </row>
@@ -649,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify validation when username field is empty</t>
+          <t>Verify login validation when username field is empty</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -667,13 +666,13 @@
         <is>
           <t>Navigate to the login page
 Leave username_textbox empty
-Enter Icstunnel1 in password_textbox
+Enter Icstunnel1 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Login submission is blocked, a validation or error indication appears for username_textbox, and the login page remains displayed without redirecting to the home page</t>
+          <t>Login request is not processed, the user remains on the login page, and a visible validation message indicates the username field is required.</t>
         </is>
       </c>
     </row>
@@ -685,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify validation when password field is empty</t>
+          <t>Verify login validation when password field is empty</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -702,14 +701,14 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in username_textbox
+Enter hacklarr into username_textbox
 Leave password_textbox empty
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Login submission is prevented, a validation or error indication appears for password_textbox, and the user remains on the login page</t>
+          <t>Login request is blocked, the login page remains displayed, and a visible validation message indicates the password field is required.</t>
         </is>
       </c>
     </row>
@@ -721,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify validation when both username and password fields are empty</t>
+          <t>Verify login validation when both username and password fields are empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -745,7 +744,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Submission is rejected, validation messages or visual error indicators appear for both fields, and the login page remains displayed without navigation</t>
+          <t>Login submission is prevented and validation messages indicate that both username and password fields are required while the login page remains visible.</t>
         </is>
       </c>
     </row>
@@ -757,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify password textbox masks entered characters</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,12 +773,13 @@
       <c r="F10" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter text into password_textbox</t>
+Click password_textbox
+Enter Icstunnel1 into password_textbox</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Characters typed into password_textbox appear masked as dots or bullet characters and the actual text value is not visible on the screen</t>
+          <t>Characters typed into password_textbox are displayed as masked characters such as dots or asterisks and the actual password text is not visible.</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify home navigation button redirects user to home page</t>
+          <t>Verify home navigation button redirects to home page</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Application navigates to the home page and the browser URL changes to http://172.21.166.115/washtabui/home</t>
+          <t>The application navigates to http://172.21.166.115/washtabui/home and the home page UI becomes visible in the browser.</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify back navigation button redirects user to home page</t>
+          <t>Verify back navigation button redirects to home page</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Application navigates away from the login page and loads the home page with URL http://172.21.166.115/washtabui/home</t>
+          <t>The application navigates away from the login page and loads the home page at http://172.21.166.115/washtabui/home.</t>
         </is>
       </c>
     </row>
@@ -859,12 +859,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify login behavior when username contains leading and trailing spaces</t>
+          <t>Verify login fails when username contains only whitespace</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -876,14 +876,14 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter space hacklarr space in username_textbox
-Enter Icstunnel1 in password_textbox
+Enter spaces into username_textbox
+Enter Icstunnel1 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>System either trims the whitespace and authenticates the user successfully redirecting to http://172.21.166.115/washtabui/home, or rejects the login attempt with a visible error while remaining on the login page</t>
+          <t>Authentication is rejected, the login page remains visible, and a validation or error message indicates the username input is invalid or empty.</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login attempt using whitespace-only values</t>
+          <t>Verify login fails when password contains only whitespace</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -912,14 +912,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter only spaces in username_textbox
-Enter only spaces in password_textbox
+Enter hacklarr into username_textbox
+Enter spaces into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>System rejects the login attempt, displays a validation or authentication error message, and remains on the login page without redirecting to the home page</t>
+          <t>Authentication attempt fails, the login page remains displayed, and a visible validation or authentication failure message appears.</t>
         </is>
       </c>
     </row>
@@ -931,7 +931,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify system behavior when SIGN IN button is clicked multiple times rapidly</t>
+          <t>Verify login behavior with leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -948,14 +948,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in username_textbox
-Enter Icstunnel1 in password_textbox
-Rapidly click sign_in_button multiple times</t>
+Enter '  hacklarr  ' into username_textbox
+Enter Icstunnel1 into password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Application processes the authentication request only once and redirects to the home page a single time without duplicate requests, page errors, or unexpected behavior</t>
+          <t>System processes the input and either trims whitespace allowing successful authentication and redirection to the home page, or rejects the login with an invalid credentials message while staying on the login page.</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login attempt with very long username and password values</t>
+          <t>Verify login attempt with very long username input</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -984,14 +984,14 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter a very long string exceeding typical username length in username_textbox
-Enter a very long string exceeding typical password length in password_textbox
+Enter a very long string exceeding normal username length into username_textbox
+Enter Icstunnel1 into password_textbox
 Click sign_in_button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Application safely rejects the authentication attempt and remains on the login page without UI breakage, application crash, or unexpected navigation</t>
+          <t>Application remains stable without UI errors, authentication is rejected, and the user remains on the login page with an invalid credentials or validation message.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify login submission using Enter key from password field</t>
+          <t>Verify login attempt with very long password input</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1020,14 +1020,14 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Enter hacklarr in username_textbox
-Enter Icstunnel1 in password_textbox
-Press Enter key while cursor focus is inside password_textbox</t>
+Enter hacklarr into username_textbox
+Enter a very long string exceeding normal password length into password_textbox
+Click sign_in_button</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pressing Enter triggers the login action and the user is successfully authenticated and redirected to http://172.21.166.115/washtabui/home</t>
+          <t>System handles the long input without UI failure, authentication is rejected, and the login page remains visible with an invalid credentials message.</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login using copy and paste for credentials</t>
+          <t>Verify multiple rapid clicks on Sign In button with valid credentials</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1056,14 +1056,122 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Navigate to the login page
-Copy the value hacklarr and paste it into username_textbox
-Copy the value Icstunnel1 and paste it into password_textbox
-Click sign_in_button</t>
+Enter hacklarr into username_textbox
+Enter Icstunnel1 into password_textbox
+Rapidly click sign_in_button multiple times</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pasted credentials are accepted as valid input and user authentication succeeds with redirection to http://172.21.166.115/washtabui/home</t>
+          <t>Only a single authentication request is processed and the user is redirected once to the home page without duplicate navigation, multiple sessions, or UI errors.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WT-LOGIN18</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Verify login using copy and paste credentials</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Copy hacklarr and paste it into username_textbox
+Copy Icstunnel1 and paste it into password_textbox
+Click sign_in_button</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Credentials pasted into the fields are accepted and authentication succeeds, redirecting the user to the home page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>WT-LOGIN19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Verify login submission using Enter key</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter hacklarr into username_textbox
+Enter Icstunnel1 into password_textbox
+Press Enter on the keyboard</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>The login form is submitted using the Enter key and successful authentication redirects the user to the home page URL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>WT-LOGIN20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Verify login attempt with special characters in username</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Navigate to the login page
+Enter user!@# into username_textbox
+Enter Icstunnel1 into password_textbox
+Click sign_in_button</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Application remains stable, authentication fails, and an invalid credentials message is displayed while the login page remains visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Generated Files 46
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -486,13 +486,18 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Navigate to http://172.21.166.115/washtabui/login?data=undefined
-Observe the login page UI</t>
+          <t>Open browser and navigate to http://172.21.166.115/washtabui/login?data=undefined
+Observe the login page layout
+Verify the username textbox is visible
+Verify the password textbox is visible
+Verify the SIGN IN button is visible
+Verify the home navigation button is visible
+Verify the back navigation button is visible</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page loads at the specified URL and username_textbox, password_textbox, sign_in_button, home_navigation_button, and back_navigation_button are visible, enabled, and ready for user interaction.</t>
+          <t>Login page loads at the specified URL and the username textbox, password textbox, SIGN IN button, home navigation button, and back navigation button are visible and enabled for interaction.</t>
         </is>
       </c>
     </row>
@@ -520,15 +525,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home where the home page UI is visible and the login page is no longer displayed.</t>
+          <t>User authentication succeeds and the browser redirects to http://172.21.166.115/washtabui/home where the home page is displayed, confirming an authenticated session.</t>
         </is>
       </c>
     </row>
@@ -540,7 +545,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify login fails with valid username and invalid password</t>
+          <t>Verify login fails with incorrect password</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,15 +561,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter WrongPassword123 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Enter WrongPassword123 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Authentication is rejected, the user remains on the login page URL, and a visible error message indicating invalid or incorrect credentials is displayed.</t>
+          <t>Authentication fails, the browser remains on the login page URL, and a visible sign-in failure message indicating invalid or incorrect credentials is displayed.</t>
         </is>
       </c>
     </row>
@@ -576,7 +581,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with invalid username and valid password</t>
+          <t>Verify login fails with incorrect username</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -592,15 +597,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter invaliduser into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter invaliduser in username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication fails, the application stays on the login page URL, and a visible message indicating invalid or incorrect credentials is displayed.</t>
+          <t>Authentication fails and the application remains on the login page without redirecting to the home page, displaying a visible authentication failure message.</t>
         </is>
       </c>
     </row>
@@ -628,15 +633,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter wronguser into username_textbox
-Enter wrongpass into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter wronguser in username textbox
+Enter wrongpassword in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails, the application remains on the login page, and a visible invalid credentials error message is shown.</t>
+          <t>Authentication fails, the user remains on the login page, and a visible error message indicates that the credentials are invalid.</t>
         </is>
       </c>
     </row>
@@ -664,15 +669,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Leave username_textbox empty
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Leave username textbox empty
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Login request is not processed, the user remains on the login page, and a visible validation message indicates the username field is required.</t>
+          <t>Login is rejected, the application remains on the login page, and a visible validation or authentication failure message appears due to missing username.</t>
         </is>
       </c>
     </row>
@@ -700,15 +705,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Leave password_textbox empty
-Click sign_in_button</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Leave password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Login request is blocked, the login page remains displayed, and a visible validation message indicates the password field is required.</t>
+          <t>Login is rejected, the user remains on the login page, and a visible validation or authentication failure message indicates that the password is missing.</t>
         </is>
       </c>
     </row>
@@ -720,7 +725,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login validation when both username and password fields are empty</t>
+          <t>Verify login validation when both username and password are empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -736,15 +741,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Leave username_textbox empty
-Leave password_textbox empty
-Click sign_in_button</t>
+          <t>Open the login page
+Leave username textbox empty
+Leave password textbox empty
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Login submission is prevented and validation messages indicate that both username and password fields are required while the login page remains visible.</t>
+          <t>Authentication is not completed and the login page remains displayed with visible feedback indicating that credentials are required.</t>
         </is>
       </c>
     </row>
@@ -772,14 +777,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Click password_textbox
-Enter Icstunnel1 into password_textbox</t>
+          <t>Open the login page
+Click the password textbox
+Enter Icstunnel1 in the password textbox</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Characters typed into password_textbox are displayed as masked characters such as dots or asterisks and the actual password text is not visible.</t>
+          <t>The password characters are masked (for example with dots or asterisks) and the actual text entered is not visible in plain text.</t>
         </is>
       </c>
     </row>
@@ -791,7 +796,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify home navigation button redirects to home page</t>
+          <t>Verify navigation to home page using home navigation button</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -807,13 +812,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Click home_navigation_button</t>
+          <t>Open the login page
+Click the home navigation button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application navigates to http://172.21.166.115/washtabui/home and the home page UI becomes visible in the browser.</t>
+          <t>The application navigates from the login page to http://172.21.166.115/washtabui/home and the home page becomes visible.</t>
         </is>
       </c>
     </row>
@@ -825,7 +830,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify back navigation button redirects to home page</t>
+          <t>Verify navigation to home page using back navigation button</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -841,8 +846,8 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Click back_navigation_button</t>
+          <t>Open the login page
+Click the back navigation button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -859,12 +864,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify login fails when username contains only whitespace</t>
+          <t>Verify username textbox accepts pasted input</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -875,15 +880,16 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter spaces into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Copy the text hacklarr to clipboard
+Open the login page
+Paste the copied value into the username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Authentication is rejected, the login page remains visible, and a validation or error message indicates the username input is invalid or empty.</t>
+          <t>The pasted value appears correctly in the username textbox and login succeeds, redirecting the user to the home page.</t>
         </is>
       </c>
     </row>
@@ -895,12 +901,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login fails when password contains only whitespace</t>
+          <t>Verify login attempt with leading and trailing spaces in username</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -911,15 +917,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter spaces into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter a username with leading and trailing spaces such as space hacklarr space in the username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Authentication attempt fails, the login page remains displayed, and a visible validation or authentication failure message appears.</t>
+          <t>Authentication fails and the application remains on the login page with a visible sign-in failure message indicating invalid credentials.</t>
         </is>
       </c>
     </row>
@@ -931,12 +937,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify login behavior with leading and trailing spaces in username</t>
+          <t>Verify login attempt with whitespace-only username</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -947,15 +953,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter '  hacklarr  ' into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter only spaces into the username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>System processes the input and either trims whitespace allowing successful authentication and redirection to the home page, or rejects the login with an invalid credentials message while staying on the login page.</t>
+          <t>Login attempt fails, the application remains on the login page, and visible feedback indicates invalid or missing username.</t>
         </is>
       </c>
     </row>
@@ -967,12 +973,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify login attempt with very long username input</t>
+          <t>Verify login attempt with whitespace-only password</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -983,15 +989,15 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter a very long string exceeding normal username length into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Enter only spaces in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Application remains stable without UI errors, authentication is rejected, and the user remains on the login page with an invalid credentials or validation message.</t>
+          <t>Authentication fails and the login page remains displayed with a visible sign-in failure message indicating invalid credentials.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1009,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify login attempt with very long password input</t>
+          <t>Verify behavior when SIGN IN button is clicked multiple times rapidly</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1019,15 +1025,15 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter a very long string exceeding normal password length into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button multiple times rapidly</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>System handles the long input without UI failure, authentication is rejected, and the login page remains visible with an invalid credentials message.</t>
+          <t>Only one authentication request is processed and the user is redirected once to the home page without duplicate navigation or UI errors.</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1045,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify multiple rapid clicks on Sign In button with valid credentials</t>
+          <t>Verify login attempt with extremely long username input</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1055,15 +1061,15 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter Icstunnel1 into password_textbox
-Rapidly click sign_in_button multiple times</t>
+          <t>Open the login page
+Enter a very long string exceeding normal username length into the username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Only a single authentication request is processed and the user is redirected once to the home page without duplicate navigation, multiple sessions, or UI errors.</t>
+          <t>The application handles the long input without UI crash, authentication fails, and the user remains on the login page with a visible sign-in failure message.</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1081,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify login using copy and paste credentials</t>
+          <t>Verify login fails with special characters in username</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1091,15 +1097,15 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Copy hacklarr and paste it into username_textbox
-Copy Icstunnel1 and paste it into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter special characters such as @@@### in the username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Credentials pasted into the fields are accepted and authentication succeeds, redirecting the user to the home page.</t>
+          <t>Authentication fails and the application remains on the login page with a visible error or sign-in failure message indicating invalid credentials.</t>
         </is>
       </c>
     </row>
@@ -1127,15 +1133,15 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter hacklarr into username_textbox
-Enter Icstunnel1 into password_textbox
-Press Enter on the keyboard</t>
+          <t>Open the login page
+Enter hacklarr in username textbox
+Enter Icstunnel1 in password textbox
+Press the Enter key on the keyboard</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>The login form is submitted using the Enter key and successful authentication redirects the user to the home page URL.</t>
+          <t>The login form is submitted using the Enter key and the user is redirected to the home page indicating successful authentication.</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1153,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Verify login attempt with special characters in username</t>
+          <t>Verify login attempt with uppercase username</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1163,15 +1169,15 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Navigate to the login page
-Enter user!@# into username_textbox
-Enter Icstunnel1 into password_textbox
-Click sign_in_button</t>
+          <t>Open the login page
+Enter HACKLARR in username textbox
+Enter Icstunnel1 in password textbox
+Click the SIGN IN button</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Application remains stable, authentication fails, and an invalid credentials message is displayed while the login page remains visible.</t>
+          <t>Authentication fails and the application remains on the login page with a visible sign-in failure message indicating invalid credentials.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Test generated files 4
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page displays all approved login controls and title</t>
+          <t>Verify login page loads with all approved UI elements visible</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,13 +486,13 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the login page URL
-Observe the login form without entering any data</t>
+          <t>Open the login page URL in the browser
+Observe the login page layout and available controls</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page title 'Login' is visible along with username textbox, password textbox, login button, and forgot password link. All controls are visible, aligned correctly, enabled for interaction, and displayed without overlap or rendering issues.</t>
+          <t>Login page title 'Login' is visible along with username textbox, password textbox, Login button, and Forgot your password? link. Username and password fields are editable, Login button is clickable, and no validation or invalid credential message is displayed on initial page load.</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login using valid username and valid password</t>
+          <t>Verify successful login using valid username and password</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -520,15 +520,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
-Enter password as 'admin123'
+          <t>Enter username as 'Admin' in the username textbox
+Enter password as 'admin123' in the password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and redirected to URL containing '/dashboard/index'. Dashboard content becomes visible and the login form is no longer displayed.</t>
+          <t>User is authenticated successfully and redirected to URL https://opensource-demo.orangehrmlive.com/web/index.php/dashboard/index. Dashboard page is displayed, login form is no longer visible, and no invalid credential message is shown.</t>
         </is>
       </c>
     </row>
@@ -540,7 +539,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify login submission using Enter key from password field with valid credentials</t>
+          <t>Verify successful login using Enter key from password field</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,15 +555,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
+          <t>Enter username as 'Admin'
 Enter password as 'admin123'
-Press Enter key while cursor is inside password textbox</t>
+Press Enter key while cursor is inside the password textbox</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Login form submits successfully using keyboard action without clicking the Login button and user is redirected to URL containing '/dashboard/index'.</t>
+          <t>Login form is submitted using keyboard action without clicking the Login button and user is redirected to the dashboard URL successfully.</t>
         </is>
       </c>
     </row>
@@ -592,15 +590,14 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'InvalidAdmin'
+          <t>Enter username as 'InvalidAdmin'
 Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Authentication is rejected, visible 'Invalid credentials' message is displayed, user remains on login page, and dashboard URL is not opened.</t>
+          <t>User remains on the login page, dashboard URL is not opened, and visible message 'Invalid credentials' is displayed near the login form.</t>
         </is>
       </c>
     </row>
@@ -628,15 +625,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
+          <t>Enter username as 'Admin'
 Enter password as 'wrongPassword123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message, dashboard page is not displayed, and login form remains accessible.</t>
+          <t>Authentication request is rejected, visible message 'Invalid credentials' is displayed, and user remains on the authentication page without dashboard access.</t>
         </is>
       </c>
     </row>
@@ -664,15 +660,14 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'WrongUser'
-Enter password as 'WrongPassword'
+          <t>Enter username as 'wrongUser'
+Enter password as 'wrongPassword'
 Click the Login button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Application displays 'Invalid credentials' message, authentication is denied, and URL remains on the login page.</t>
+          <t>Login attempt fails with visible 'Invalid credentials' message, login page remains displayed, and dashboard page is not opened.</t>
         </is>
       </c>
     </row>
@@ -684,7 +679,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify required validation when username and password fields are empty</t>
+          <t>Verify required validation when username and password are left empty</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -700,14 +695,14 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the login page
-Leave username and password fields empty
+          <t>Keep username textbox empty
+Keep password textbox empty
 Click the Login button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Required validation messages are displayed for username and password fields, login request is not submitted, and user remains on login page.</t>
+          <t>Validation message 'Required' is displayed for both username and password fields. Login request is not submitted and user remains on login page.</t>
         </is>
       </c>
     </row>
@@ -719,7 +714,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify required validation when password field is empty</t>
+          <t>Verify required validation when username is empty and password is entered</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -735,15 +730,14 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
-Leave password field empty
+          <t>Leave username textbox empty
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Password field displays required validation message, authentication request is blocked, and dashboard page is not opened.</t>
+          <t>Validation message 'Required' is displayed for username field only. Login request is blocked and dashboard page is not opened.</t>
         </is>
       </c>
     </row>
@@ -755,7 +749,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify required validation when username field is empty</t>
+          <t>Verify required validation when password is empty and username is entered</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -771,15 +765,14 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the login page
-Leave username field empty
-Enter password as 'admin123'
+          <t>Enter username as 'Admin'
+Leave password textbox empty
 Click the Login button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Username field displays required validation message, login submission is prevented, and user remains on the login page.</t>
+          <t>Validation message 'Required' is displayed for password field only. User remains on login page and authentication request is not processed.</t>
         </is>
       </c>
     </row>
@@ -791,7 +784,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify password characters are masked while typing</t>
+          <t>Verify password field masks entered characters</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -807,13 +800,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the login page
-Type password text into the password textbox</t>
+          <t>Click inside password textbox
+Type password value 'admin123'</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Typed password characters are masked with hidden symbols and actual password text is not visible on screen.</t>
+          <t>Password field masks all entered characters with hidden or bullet-style characters and actual password text is not visible on screen.</t>
         </is>
       </c>
     </row>
@@ -825,12 +818,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify forgot password link is visible and navigates to password recovery page</t>
+          <t>Verify username field handling of leading and trailing spaces</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -841,13 +834,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the login page
-Click the Forgot your password link</t>
+          <t>Enter username as '  Admin  '
+Enter password as 'admin123'
+Click the Login button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>User is redirected away from the login page to a password recovery or reset page and recovery-related page content becomes visible.</t>
+          <t>Application processes the username input consistently. User either logs in successfully after trimming spaces or receives a visible authentication rejection message without UI breakage, page crash, or frozen controls.</t>
         </is>
       </c>
     </row>
@@ -859,12 +853,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify logout redirects authenticated user back to login page</t>
+          <t>Verify login behavior when password contains leading and trailing spaces</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -875,15 +869,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the login page
-Login using valid credentials
-Click the user profile menu in the application header
-Click Logout option</t>
+          <t>Enter username as 'Admin'
+Enter password as '  admin123  '
+Click the Login button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Authenticated session is terminated, application redirects to the login page URL, and username textbox, password textbox, and Login button are visible again.</t>
+          <t>Authentication fails with visible 'Invalid credentials' message if spaces are treated as part of the password value. User remains on login page and dashboard URL is not opened.</t>
         </is>
       </c>
     </row>
@@ -895,12 +888,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify login behavior with leading and trailing spaces in username field</t>
+          <t>Verify whitespace-only values are not accepted in username and password fields</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -911,15 +904,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as '  Admin  '
-Enter password as 'admin123'
+          <t>Enter only spaces in username textbox
+Enter only spaces in password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Application handles leading and trailing spaces consistently by either authenticating successfully after trimming spaces or displaying visible authentication failure feedback. No broken layout, script error, or blank page appears.</t>
+          <t>Login is not successful. User remains on login page and either validation message 'Required' or message 'Invalid credentials' is displayed without navigation to dashboard page.</t>
         </is>
       </c>
     </row>
@@ -931,7 +923,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify password field treats leading and trailing spaces as part of password value</t>
+          <t>Verify username field accepts pasted text input</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -947,15 +939,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
-Enter password as '  admin123  '
+          <t>Copy the value 'Admin' from an external source
+Paste the value into username textbox
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message because password value containing surrounding spaces does not match the stored password.</t>
+          <t>Pasted username value is accepted correctly, login request is processed successfully, and dashboard page is displayed after authentication.</t>
         </is>
       </c>
     </row>
@@ -967,12 +959,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify whitespace-only input is rejected in username and password fields</t>
+          <t>Verify password field accepts pasted text input securely</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -983,15 +975,14 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter only spaces into username textbox
-Enter only spaces into password textbox
+          <t>Enter username as 'Admin'
+Paste 'admin123' into password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>User is not authenticated, validation or invalid credential feedback is displayed, and application remains on login page without dashboard navigation.</t>
+          <t>Pasted password remains masked in the password field and user is authenticated successfully without exposing the pasted password text.</t>
         </is>
       </c>
     </row>
@@ -1003,12 +994,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify login is case-sensitive for username field</t>
+          <t>Verify login button behavior on repeated rapid clicks</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1019,15 +1010,13 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'admin'
-Enter password as 'admin123'
-Click the Login button</t>
+          <t>Enter valid username and password
+Click the Login button repeatedly multiple times in quick succession</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message because username case does not match the valid credential.</t>
+          <t>Application processes only one successful login session, redirects once to the dashboard page, and does not display duplicate requests, duplicate sessions, browser errors, or broken UI behavior.</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1028,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify login is case-sensitive for password field</t>
+          <t>Verify username field handles very long input gracefully</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1055,15 +1044,14 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
-Enter password as 'Admin123'
+          <t>Enter a username value significantly longer than expected normal length
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message because password case does not match the valid password.</t>
+          <t>Application remains responsive, login page layout does not break, and authentication is rejected with visible validation or invalid credentials message without browser crash.</t>
         </is>
       </c>
     </row>
@@ -1075,12 +1063,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify special characters in username field are rejected</t>
+          <t>Verify password field handles very long input gracefully</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1091,15 +1079,14 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as '@@@###$$$'
-Enter password as 'admin123'
+          <t>Enter username as 'Admin'
+Enter a password value significantly longer than expected normal length
 Click the Login button</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Login attempt is rejected with visible authentication failure feedback and dashboard page is not opened.</t>
+          <t>Application remains stable and responsive, password field continues masking input, and authentication is rejected without layout corruption or application error.</t>
         </is>
       </c>
     </row>
@@ -1111,12 +1098,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Verify very long username and password inputs do not break login form</t>
+          <t>Verify login is case sensitive for username</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1127,15 +1114,14 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Open the login page
-Paste a very long string into username textbox
-Paste a very long string into password textbox
+          <t>Enter username as 'admin'
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Application remains responsive, input fields continue functioning without layout corruption, and authentication failure is handled gracefully without browser crash or application error.</t>
+          <t>Authentication fails with visible 'Invalid credentials' message and user remains on login page when incorrect username case is entered.</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1133,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Verify repeated clicking of Login button with valid credentials does not create duplicate navigation behavior</t>
+          <t>Verify login is case sensitive for password</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1163,15 +1149,14 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'Admin'
-Enter password as 'admin123'
-Rapidly click the Login button multiple times</t>
+          <t>Enter username as 'Admin'
+Enter password as 'ADMIN123'
+Click the Login button</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Only one authenticated session is created, user is redirected once to dashboard page, and no duplicate page loads, duplicate sessions, or UI instability occurs.</t>
+          <t>Authentication fails with visible 'Invalid credentials' message because password case does not match the valid credential value.</t>
         </is>
       </c>
     </row>
@@ -1183,12 +1168,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Verify repeated clicking of Login button with invalid credentials consistently shows rejection</t>
+          <t>Verify special characters in username field are rejected during login</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1199,15 +1184,14 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Open the login page
-Enter username as 'InvalidAdmin'
-Enter password as 'wrongPassword'
-Rapidly click the Login button multiple times</t>
+          <t>Enter username as '@@@###'
+Enter password as 'admin123'
+Click the Login button</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Application consistently rejects authentication, displays invalid credential feedback without duplicated error overlays, and remains stable on login page.</t>
+          <t>Login fails with visible 'Invalid credentials' message and user stays on login page without navigation to dashboard.</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1203,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Verify copy-paste of valid credentials into login fields authenticates successfully</t>
+          <t>Verify special characters in password field do not break authentication flow</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1235,15 +1219,14 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Open the login page
-Copy and paste 'Admin' into username textbox
-Copy and paste 'admin123' into password textbox
+          <t>Enter username as 'Admin'
+Enter password as '@@@###$$$'
 Click the Login button</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Pasted credentials are accepted correctly, authentication succeeds, and user is redirected to URL containing '/dashboard/index'.</t>
+          <t>Authentication is rejected with visible 'Invalid credentials' message and login page continues functioning normally without UI or browser errors.</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1238,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Verify login page remains accessible after failed login attempt</t>
+          <t>Verify Forgot your password link navigation</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1272,13 +1255,12 @@
       <c r="F24" t="inlineStr">
         <is>
           <t>Open the login page
-Attempt login using invalid credentials
-Observe the login page after error message appears</t>
+Click the 'Forgot your password?' link</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Username textbox, password textbox, Login button, and Forgot your password link remain visible, enabled, and usable after failed authentication attempt.</t>
+          <t>User is redirected from the login page to the password recovery workflow page and login form is no longer displayed.</t>
         </is>
       </c>
     </row>
@@ -1290,12 +1272,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Verify browser refresh on login page preserves application usability</t>
+          <t>Verify successful logout returns user to login page</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1306,15 +1288,14 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Open the login page
-Refresh the browser page
-Observe the login form
-Login using valid credentials</t>
+          <t>Login using valid credentials
+Click on the logged-in user menu
+Click the Logout option</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Login page reloads successfully with all approved controls visible, and valid authentication after refresh redirects user to dashboard page successfully.</t>
+          <t>Authenticated session is terminated successfully and application redirects back to the login page URL with username textbox, password textbox, and Login button visible again.</t>
         </is>
       </c>
     </row>
@@ -1326,12 +1307,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Verify login button is visible and clickable on initial page load</t>
+          <t>Verify invalid credential message disappears after successful login attempt</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1342,14 +1323,14 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Open the login page
-Observe the Login button
-Click the Login button without entering credentials</t>
+          <t>Attempt login with invalid credentials and observe the invalid credentials message
+Correct the username and password using valid credentials
+Click the Login button</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Login button is visible and clickable, and clicking it without credentials displays required validation messages for mandatory fields.</t>
+          <t>Previously displayed invalid credentials message is cleared after successful authentication and user is redirected to the dashboard page.</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1342,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Verify user cannot access dashboard URL directly after logout</t>
+          <t>Verify tab navigation order on login page</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1377,15 +1358,83 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Open the login page
-Login using valid credentials
-Logout from the application
-Manually enter the dashboard URL in browser address bar</t>
+          <t>Place cursor on username textbox
+Press Tab key repeatedly to navigate through interactive controls</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Application redirects user back to the login page or blocks access to dashboard content because the authenticated session has ended.</t>
+          <t>Keyboard focus moves sequentially from username textbox to password textbox to Login button and then to Forgot your password? link without skipping controls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>WT-LOGIN27</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Verify login page remains accessible after failed login attempt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Enter invalid credentials
+Click the Login button
+Observe page state after error message appears</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Username textbox, password textbox, Login button, and Forgot your password? link remain visible, enabled, and usable after failed authentication attempt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>WT-LOGIN28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Verify username and password field behavior after invalid login attempt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Enter invalid username and password values
+Click the Login button
+Observe the values displayed in username and password fields after the error message appears</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Username field retains the entered username value after failed login attempt while password field remains masked or is cleared according to application behavior. Invalid credentials message remains visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Committing Test generated files 5
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify login page loads with all approved UI elements visible</t>
+          <t>Verify login page displays all required login controls and labels</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,12 +487,12 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Open the login page URL in the browser
-Observe the login page layout and available controls</t>
+Observe the login form area without entering any data</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Login page title 'Login' is visible along with username textbox, password textbox, Login button, and Forgot your password? link. Username and password fields are editable, Login button is clickable, and no validation or invalid credential message is displayed on initial page load.</t>
+          <t>Login page heading 'Login' is visible. Username textbox, password textbox, Login button, and Forgot your password? link are displayed, enabled, and accessible for interaction.</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify successful login using valid username and password</t>
+          <t>Verify successful login using valid username and valid password</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -520,14 +520,15 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin' in the username textbox
-Enter password as 'admin123' in the password textbox
+          <t>Open the login page
+Enter username as 'Admin'
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>User is authenticated successfully and redirected to URL https://opensource-demo.orangehrmlive.com/web/index.php/dashboard/index. Dashboard page is displayed, login form is no longer visible, and no invalid credential message is shown.</t>
+          <t>User is authenticated successfully and redirected to URL https://opensource-demo.orangehrmlive.com/web/index.php/dashboard/index. Dashboard page is displayed and login form is no longer visible.</t>
         </is>
       </c>
     </row>
@@ -539,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify successful login using Enter key from password field</t>
+          <t>Verify successful login when credentials are pasted into the fields</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -555,14 +556,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter password as 'admin123'
-Press Enter key while cursor is inside the password textbox</t>
+          <t>Open the login page
+Copy and paste 'Admin' into the username textbox
+Copy and paste 'admin123' into the password textbox
+Click the Login button</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Login form is submitted using keyboard action without clicking the Login button and user is redirected to the dashboard URL successfully.</t>
+          <t>Pasted values are accepted without truncation or formatting issues and user is redirected successfully to the dashboard URL after clicking Login.</t>
         </is>
       </c>
     </row>
@@ -574,12 +576,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify login fails with invalid username and valid password</t>
+          <t>Verify login can be submitted using Enter key from password field</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -590,14 +592,15 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Enter username as 'InvalidAdmin'
-Enter password as 'admin123'
-Click the Login button</t>
+          <t>Open the login page
+Enter valid username 'Admin'
+Enter valid password 'admin123'
+Press the Enter key while focused on the password textbox</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>User remains on the login page, dashboard URL is not opened, and visible message 'Invalid credentials' is displayed near the login form.</t>
+          <t>Login form is submitted through keyboard interaction and user is redirected to the dashboard page without clicking the Login button.</t>
         </is>
       </c>
     </row>
@@ -609,7 +612,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify login fails with valid username and invalid password</t>
+          <t>Verify login fails with invalid username and valid password</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -625,14 +628,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter password as 'wrongPassword123'
+          <t>Open the login page
+Enter username as 'InvalidAdmin'
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication request is rejected, visible message 'Invalid credentials' is displayed, and user remains on the authentication page without dashboard access.</t>
+          <t>User remains on the login page, dashboard URL is not opened, and 'Invalid credentials' message is displayed below or near the login form.</t>
         </is>
       </c>
     </row>
@@ -644,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify login fails with both username and password invalid</t>
+          <t>Verify login fails with valid username and invalid password</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -660,14 +664,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Enter username as 'wrongUser'
-Enter password as 'wrongPassword'
+          <t>Open the login page
+Enter username as 'Admin'
+Enter password as 'wrongpassword'
 Click the Login button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Login attempt fails with visible 'Invalid credentials' message, login page remains displayed, and dashboard page is not opened.</t>
+          <t>Authentication is rejected, user stays on the login page, and visible 'Invalid credentials' message is displayed without redirecting to dashboard.</t>
         </is>
       </c>
     </row>
@@ -679,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify required validation when username and password are left empty</t>
+          <t>Verify login fails with both invalid username and invalid password</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -695,14 +700,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Keep username textbox empty
-Keep password textbox empty
+          <t>Open the login page
+Enter username as 'wronguser'
+Enter password as 'wrongpassword'
 Click the Login button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Validation message 'Required' is displayed for both username and password fields. Login request is not submitted and user remains on login page.</t>
+          <t>Login attempt is rejected, 'Invalid credentials' message is displayed, login form remains visible, and dashboard page is not loaded.</t>
         </is>
       </c>
     </row>
@@ -714,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify required validation when username is empty and password is entered</t>
+          <t>Verify required validation when username and password fields are empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -730,14 +736,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Leave username textbox empty
-Enter password as 'admin123'
+          <t>Open the login page
+Leave username textbox empty
+Leave password textbox empty
 Click the Login button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Validation message 'Required' is displayed for username field only. Login request is blocked and dashboard page is not opened.</t>
+          <t>Required validation messages are displayed for both username and password fields. Login form is not submitted and user remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -749,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify required validation when password is empty and username is entered</t>
+          <t>Verify required validation when username is empty and password is entered</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -765,14 +772,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Leave password textbox empty
+          <t>Open the login page
+Leave username textbox empty
+Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Validation message 'Required' is displayed for password field only. User remains on login page and authentication request is not processed.</t>
+          <t>Required validation message is displayed for the username field only and authentication does not proceed.</t>
         </is>
       </c>
     </row>
@@ -784,12 +792,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters</t>
+          <t>Verify required validation when password is empty and username is entered</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -800,13 +808,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Click inside password textbox
-Type password value 'admin123'</t>
+          <t>Open the login page
+Enter username as 'Admin'
+Leave password textbox empty
+Click the Login button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Password field masks all entered characters with hidden or bullet-style characters and actual password text is not visible on screen.</t>
+          <t>Required validation message is displayed for the password field only and user remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -818,7 +828,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify username field handling of leading and trailing spaces</t>
+          <t>Verify login behavior with leading and trailing spaces in username field</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -834,14 +844,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Enter username as '  Admin  '
+          <t>Open the login page
+Enter username as '  Admin  '
 Enter password as 'admin123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Application processes the username input consistently. User either logs in successfully after trimming spaces or receives a visible authentication rejection message without UI breakage, page crash, or frozen controls.</t>
+          <t>Application handles leading and trailing spaces consistently by either trimming the username and authenticating successfully or rejecting the login with visible validation or invalid credential feedback. No broken UI or application error is displayed.</t>
         </is>
       </c>
     </row>
@@ -853,12 +864,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify login behavior when password contains leading and trailing spaces</t>
+          <t>Verify login fails when only whitespace is entered in username and password fields</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -869,14 +880,15 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter password as '  admin123  '
+          <t>Open the login page
+Enter only spaces into the username textbox
+Enter only spaces into the password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message if spaces are treated as part of the password value. User remains on login page and dashboard URL is not opened.</t>
+          <t>User is not authenticated, dashboard page is not opened, and application displays either Required validation messages or Invalid credentials message while keeping the login form visible.</t>
         </is>
       </c>
     </row>
@@ -888,12 +900,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify whitespace-only values are not accepted in username and password fields</t>
+          <t>Verify password characters remain masked while typing</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -904,14 +916,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Enter only spaces in username textbox
-Enter only spaces in password textbox
-Click the Login button</t>
+          <t>Open the login page
+Type 'admin123' into the password textbox</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Login is not successful. User remains on login page and either validation message 'Required' or message 'Invalid credentials' is displayed without navigation to dashboard page.</t>
+          <t>Password field masks entered characters and the actual password text is not readable on screen while typing.</t>
         </is>
       </c>
     </row>
@@ -923,12 +934,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify username field accepts pasted text input</t>
+          <t>Verify forgot password link navigates to password recovery page</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -939,15 +950,13 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Copy the value 'Admin' from an external source
-Paste the value into username textbox
-Enter password as 'admin123'
-Click the Login button</t>
+          <t>Open the login page
+Click the 'Forgot your password?' link</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pasted username value is accepted correctly, login request is processed successfully, and dashboard page is displayed after authentication.</t>
+          <t>User is redirected from the login page to the password recovery workflow page and the login form is no longer the active screen.</t>
         </is>
       </c>
     </row>
@@ -959,7 +968,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify password field accepts pasted text input securely</t>
+          <t>Verify keyboard Tab navigation moves focus through login controls in sequence</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -975,14 +984,13 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Paste 'admin123' into password textbox
-Click the Login button</t>
+          <t>Open the login page
+Press the Tab key repeatedly to navigate through interactive controls</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pasted password remains masked in the password field and user is authenticated successfully without exposing the pasted password text.</t>
+          <t>Keyboard focus moves sequentially through username textbox, password textbox, Login button, and Forgot your password? link in a usable navigation order. Focused controls are visibly active and operable using keyboard input.</t>
         </is>
       </c>
     </row>
@@ -994,12 +1002,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify login button behavior on repeated rapid clicks</t>
+          <t>Verify login is case-sensitive for username credentials</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1010,13 +1018,15 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Enter valid username and password
-Click the Login button repeatedly multiple times in quick succession</t>
+          <t>Open the login page
+Enter username as 'admin'
+Enter password as 'admin123'
+Click the Login button</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Application processes only one successful login session, redirects once to the dashboard page, and does not display duplicate requests, duplicate sessions, browser errors, or broken UI behavior.</t>
+          <t>Authentication fails because username case does not match the valid credential. 'Invalid credentials' message is displayed and dashboard page is not opened.</t>
         </is>
       </c>
     </row>
@@ -1028,12 +1038,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify username field handles very long input gracefully</t>
+          <t>Verify login is case-sensitive for password credentials</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1044,14 +1054,15 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Enter a username value significantly longer than expected normal length
-Enter password as 'admin123'
+          <t>Open the login page
+Enter username as 'Admin'
+Enter password as 'ADMIN123'
 Click the Login button</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Application remains responsive, login page layout does not break, and authentication is rejected with visible validation or invalid credentials message without browser crash.</t>
+          <t>Authentication fails because password case does not match the valid credential. 'Invalid credentials' message is displayed and user remains on the login page.</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1074,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify password field handles very long input gracefully</t>
+          <t>Verify login behavior with very long username and password values</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1079,14 +1090,15 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter a password value significantly longer than expected normal length
+          <t>Open the login page
+Enter a very long string exceeding normal credential length into the username textbox
+Enter a very long string exceeding normal credential length into the password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Application remains stable and responsive, password field continues masking input, and authentication is rejected without layout corruption or application error.</t>
+          <t>Application handles oversized input without UI distortion, browser crash, or server error. User is not authenticated and login page remains functional after submission.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1110,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Verify login is case sensitive for username</t>
+          <t>Verify login fails when special characters are entered in username and password fields</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1114,14 +1126,15 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Enter username as 'admin'
-Enter password as 'admin123'
+          <t>Open the login page
+Enter special characters into the username textbox
+Enter special characters into the password textbox
 Click the Login button</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message and user remains on login page when incorrect username case is entered.</t>
+          <t>Authentication is rejected, login page remains displayed, and visible invalid credential feedback is shown without application crash or script error.</t>
         </is>
       </c>
     </row>
@@ -1133,12 +1146,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Verify login is case sensitive for password</t>
+          <t>Verify repeated clicking on Login button with valid credentials does not create duplicate login actions</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1149,14 +1162,15 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter password as 'ADMIN123'
-Click the Login button</t>
+          <t>Open the login page
+Enter valid username 'Admin'
+Enter valid password 'admin123'
+Rapidly click the Login button multiple times</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Authentication fails with visible 'Invalid credentials' message because password case does not match the valid credential value.</t>
+          <t>Application processes only a single authenticated session, redirects user once to the dashboard page, and no duplicate requests, UI freezes, or error messages are visible.</t>
         </is>
       </c>
     </row>
@@ -1168,12 +1182,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Verify special characters in username field are rejected during login</t>
+          <t>Verify logout returns authenticated user back to login page</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1184,14 +1198,14 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Enter username as '@@@###'
-Enter password as 'admin123'
-Click the Login button</t>
+          <t>Login using valid credentials
+Click the user profile menu
+Click the Logout option</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Login fails with visible 'Invalid credentials' message and user stays on login page without navigation to dashboard.</t>
+          <t>Authenticated session is terminated, user is redirected to the login page URL, and username textbox, password textbox, and Login button are visible again.</t>
         </is>
       </c>
     </row>
@@ -1203,12 +1217,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Verify special characters in password field do not break authentication flow</t>
+          <t>Verify invalid credential message disappears after successful login retry</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1219,14 +1233,17 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Enter username as 'Admin'
-Enter password as '@@@###$$$'
-Click the Login button</t>
+          <t>Open the login page
+Attempt login using invalid credentials
+Verify the invalid credentials message is displayed
+Replace the username with 'Admin'
+Replace the password with 'admin123'
+Click the Login button again</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Authentication is rejected with visible 'Invalid credentials' message and login page continues functioning normally without UI or browser errors.</t>
+          <t>Previous invalid credentials message is cleared after successful authentication and user is redirected to the dashboard page successfully.</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1255,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Verify Forgot your password link navigation</t>
+          <t>Verify browser refresh on login page retains stable login form state</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1255,12 +1272,12 @@
       <c r="F24" t="inlineStr">
         <is>
           <t>Open the login page
-Click the 'Forgot your password?' link</t>
+Refresh the browser page</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>User is redirected from the login page to the password recovery workflow page and login form is no longer displayed.</t>
+          <t>Login page reloads successfully and username textbox, password textbox, Login button, and Forgot your password? link remain visible, enabled, and usable after refresh.</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1289,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Verify successful logout returns user to login page</t>
+          <t>Verify login button is clickable and responsive on page load</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1288,153 +1305,14 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Login using valid credentials
-Click on the logged-in user menu
-Click the Logout option</t>
+          <t>Open the login page
+Observe the Login button before entering any data
+Click the Login button</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Authenticated session is terminated successfully and application redirects back to the login page URL with username textbox, password textbox, and Login button visible again.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>WT-LOGIN25</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Verify invalid credential message disappears after successful login attempt</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Attempt login with invalid credentials and observe the invalid credentials message
-Correct the username and password using valid credentials
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Previously displayed invalid credentials message is cleared after successful authentication and user is redirected to the dashboard page.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>WT-LOGIN26</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Verify tab navigation order on login page</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>Place cursor on username textbox
-Press Tab key repeatedly to navigate through interactive controls</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Keyboard focus moves sequentially from username textbox to password textbox to Login button and then to Forgot your password? link without skipping controls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>WT-LOGIN27</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Verify login page remains accessible after failed login attempt</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Enter invalid credentials
-Click the Login button
-Observe page state after error message appears</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Username textbox, password textbox, Login button, and Forgot your password? link remain visible, enabled, and usable after failed authentication attempt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>WT-LOGIN28</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Verify username and password field behavior after invalid login attempt</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Enter invalid username and password values
-Click the Login button
-Observe the values displayed in username and password fields after the error message appears</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Username field retains the entered username value after failed login attempt while password field remains masked or is cleared according to application behavior. Invalid credentials message remains visible.</t>
+          <t>Login button is visible and clickable on page load. Clicking without credentials triggers required field validation messages without page crash or unresponsive behavior.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 14
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Open Login page from Home page using person/profile button</t>
+          <t>Verify Login page opens from Home page using the person/profile button</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page is displayed in guest state
+          <t>Navigate to http://localhost/washtabui/home
+Verify the application is displayed in guest state
 Click the person/profile button on the Home page</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Login page opens from the Home page and displays Username field, Password field, Login button, Back button, and Home button in an interactive state.</t>
+          <t>The Login page/view opens from the Home page and displays Username field, Password field, Login button, Back button, and Home button in an interactive state.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and enabled after opening Login page</t>
+          <t>Verify Login page controls are visible and enabled after navigation from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,14 +521,14 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to the Home page in guest state
-Click the person/profile button to open the Login page
-Observe the Login page controls without entering data</t>
+          <t>Open the Home page in guest state
+Click the person/profile button to open Login page
+Inspect the Login page controls</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Username field, Password field, Login button, Back button, and Home button are visible and enabled for user interaction on the Login page.</t>
+          <t>Username field, Password field, Login button, Back button, and Home button are visible, enabled, and available for interaction on the Login page.</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password input is masked while typing password characters</t>
+          <t>Verify password field masks entered characters by default</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,12 +558,12 @@
         <is>
           <t>Open the Login page from the Home page
 Click inside the Password field
-Type the password value Carwash#1 into the Password field</t>
+Type the password value Carwash#1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered password characters and does not display the plain text password value on screen.</t>
+          <t>The Password field masks all entered characters and does not display the raw password text on screen.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Login successfully using approved valid credentials</t>
+          <t>Verify successful login using approved valid credentials returns user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -592,14 +592,14 @@
       <c r="F5" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
-Enter Carwash#1 into the Password field
+Enter username krisadmin in the Username field
+Enter password Carwash#1 in the Password field
 Click the Login button</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, replaces the guest person/profile button with the logged-in user name, and displays authenticated-only features.</t>
+          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, replaces the person/profile button with the logged-in user name, and displays authenticated-only features.</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify failed login with invalid username and valid password</t>
+          <t>Verify invalid username prevents authentication and displays login error</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -628,14 +628,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter invaliduser into the Username field
-Enter Carwash#1 into the Password field
+Enter invalid username invaliduser
+Enter valid password Carwash#1
 Click the Login button</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails, an error message is displayed, the user remains unauthenticated, and the Login page remains visible without transition to authenticated Home state.</t>
+          <t>Authentication fails, an observable login error message is displayed, the application remains unauthenticated, and the user stays on the Login page or in guest state.</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify failed login with valid username and invalid password</t>
+          <t>Verify invalid password prevents authentication and displays login error</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -664,14 +664,14 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
-Enter InvalidPass123 into the Password field
+Enter valid username krisadmin
+Enter invalid password WrongPassword1
 Click the Login button</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, an error message is displayed, the Login page remains open, and the Home page does not transition into authenticated state.</t>
+          <t>Authentication fails, an observable login error message is displayed, the application remains unauthenticated, and the Login page remains active.</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify failed login with both username and password invalid</t>
+          <t>Verify login attempt with both invalid username and invalid password is rejected</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -700,14 +700,14 @@
       <c r="F8" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter invaliduser into the Username field
-Enter InvalidPass123 into the Password field
+Enter invalid username wronguser
+Enter invalid password wrongpass
 Click the Login button</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication is rejected with visible error feedback and the user remains on the Login page in unauthenticated state.</t>
+          <t>Authentication is rejected, visible error feedback is displayed, and the user is not redirected to authenticated Home state.</t>
         </is>
       </c>
     </row>
@@ -719,7 +719,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify required field validation when Login is clicked with both fields empty</t>
+          <t>Verify required field validation when Login button is clicked with both fields empty</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -736,13 +736,13 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Leave the Username and Password fields empty
+Leave Username and Password fields empty
 Click the Login button</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Required field validation messages are displayed for Username and Password and authentication does not proceed.</t>
+          <t>Required field validation is displayed for Username and Password fields and authentication does not proceed.</t>
         </is>
       </c>
     </row>
@@ -772,13 +772,13 @@
         <is>
           <t>Open the Login page from the Home page
 Leave the Username field empty
-Enter Carwash#1 into the Password field
+Enter password Carwash#1 in the Password field
 Click the Login button</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>A visible validation message is shown for the required Username field and login is blocked without leaving the Login page.</t>
+          <t>A visible Username required validation message is displayed and login does not proceed.</t>
         </is>
       </c>
     </row>
@@ -807,14 +807,14 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
+Enter username krisadmin in the Username field
 Leave the Password field empty
 Click the Login button</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>A visible validation message is shown for the required Password field and login does not proceed.</t>
+          <t>A visible Password required validation message is displayed and login does not proceed.</t>
         </is>
       </c>
     </row>
@@ -826,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify login behavior with leading and trailing spaces in both valid credential fields</t>
+          <t>Verify Back button on Login page returns user to Home page guest state</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -843,14 +843,12 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter value with spaces around the username as  krisadmin
-Enter value with spaces around the password as  Carwash#1
-Click the Login button</t>
+Click the Back button</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application handles leading and trailing spaces according to business behavior and the observed authentication result is consistent and visibly validated on screen.</t>
+          <t>The application returns to the Home page in guest state and the Login page is no longer displayed.</t>
         </is>
       </c>
     </row>
@@ -862,12 +860,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify login rejection with whitespace-only Username and Password values</t>
+          <t>Verify Home button on Login page returns user to Home page guest state</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -879,14 +877,12 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter only spaces into the Username field
-Enter only spaces into the Password field
-Click the Login button</t>
+Click the Home button</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Whitespace-only values are rejected, required or validation feedback is displayed, and the user remains on the Login page without authentication.</t>
+          <t>The application returns to the Home page in guest state and the Login page is closed.</t>
         </is>
       </c>
     </row>
@@ -898,7 +894,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Username field accepts pasted valid value and authenticates successfully</t>
+          <t>Verify leading and trailing spaces in valid username and password are handled during login</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -915,14 +911,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Paste krisadmin into the Username field
-Enter Carwash#1 into the Password field
+Enter username with leading and trailing spaces as '  krisadmin  '
+Enter password with leading and trailing spaces as '  Carwash#1  '
 Click the Login button</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The pasted Username value is accepted correctly and the user is authenticated successfully to the Home page authenticated state.</t>
+          <t>The application handles leading and trailing spaces according to business behavior, with either successful authentication after trimming valid values or visible rejection feedback while remaining unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -934,12 +930,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify Password field accepts pasted password while remaining masked</t>
+          <t>Verify whitespace-only Username and Password values are not accepted</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -951,15 +947,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
-Paste Carwash#1 into the Password field
-Observe the Password field display
+Enter only spaces in the Username field
+Enter only spaces in the Password field
 Click the Login button</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The pasted password remains masked in the Password field and the valid credentials authenticate the user successfully.</t>
+          <t>Whitespace-only values are rejected, required or invalid input validation is displayed, and the application does not authenticate the user.</t>
         </is>
       </c>
     </row>
@@ -971,12 +966,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user from Login page to Home page</t>
+          <t>Verify special characters in invalid credentials do not bypass authentication</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -988,12 +983,14 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Click the Back button on the Login page</t>
+Enter username krisadmin@@
+Enter password Carwash#1!!
+Click the Login button</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The user is returned to the Home page in guest state after clicking the Back button.</t>
+          <t>The invalid credential values are rejected, authentication does not occur, and an observable login failure message is displayed.</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1002,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user from Login page to Home page</t>
+          <t>Verify long Username and Password input values are handled without application crash</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1022,12 +1019,14 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Click the Home button on the Login page</t>
+Enter an excessively long value into the Username field
+Enter an excessively long value into the Password field
+Click the Login button</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The user is returned to the Home page in guest state after clicking the Home button.</t>
+          <t>The Login page remains stable, authentication is rejected for invalid long credentials, and visible feedback or validation is displayed without UI corruption.</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1038,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Verify authenticated-only features become available after successful login</t>
+          <t>Verify user remains in guest state after failed authentication attempt</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1056,15 +1055,15 @@
       <c r="F18" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
-Enter Carwash#1 into the Password field
+Enter invalid username invaliduser
+Enter invalid password invalidpass
 Click the Login button
-Inspect the Home page after authentication</t>
+Navigate back to the Home page if still on Login page</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Authenticated-only features become available on the Home page and the logged-in user name replaces the guest person/profile control.</t>
+          <t>The application remains in guest state, authenticated-user UI is not displayed, and the person/profile button remains visible instead of a logged-in user name.</t>
         </is>
       </c>
     </row>
@@ -1076,12 +1075,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Verify invalid login does not transition away from Login page</t>
+          <t>Verify authenticated Home page displays logged-in user identity after successful login</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1093,124 +1092,15 @@
       <c r="F19" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page
-Enter invaliduser into the Username field
-Enter wrongpassword into the Password field
+Enter username krisadmin
+Enter password Carwash#1
 Click the Login button
-Observe the current page state</t>
+Observe the Home page after authentication</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>The application remains on the Login page after failed authentication and no authenticated Home page UI is displayed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>WT-LOGIN19</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Verify username value remains unchanged after failed authentication attempt</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page
-Enter krisadmin into the Username field
-Enter invalidpassword into the Password field
-Click the Login button
-Observe the Username field after login failure</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>The Login page remains visible after authentication failure and the Username field value remains displayed for correction while the user stays unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>WT-LOGIN20</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Verify special characters in Username field do not authenticate invalid user</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page
-Enter krisadmin@@@ into the Username field
-Enter Carwash#1 into the Password field
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Authentication is rejected with visible error feedback and the application remains in unauthenticated Login state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>WT-LOGIN21</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Verify very long Username and Password values are handled without application crash</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page
-Enter a very long text value exceeding normal username length into the Username field
-Enter a very long text value exceeding normal password length into the Password field
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>The application handles oversized input safely by rejecting authentication or showing validation feedback without page crash, broken layout, or unintended authenticated access.</t>
+          <t>The authenticated Home page displays the logged-in user name in place of the person/profile button and exposes authenticated-only functionality.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 19
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Login page opens from Home page using the Person/Profile button</t>
+          <t>Verify unauthenticated guest user can open the Login page from the Home page person/profile button</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home
-Verify the Home page is displayed in guest state
-Click the Person/Profile button on the Home page</t>
+          <t>Open the WashTab application and navigate to http://localhost/washtabui/home.
+Verify the Home page is displayed in guest state without authenticated user identity visible.
+Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The Login page opens from the Home page and displays the Username field, Password field, Login button, Back button, and Home button in an interactive state.</t>
+          <t>The application transitions from the guest Home page to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactive.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and enabled after navigation from Home page</t>
+          <t>Verify Login page controls are visible and enabled after opening Login page from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,9 +521,9 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state
-Click the Person/Profile button to open the Login page
-Observe the Login page controls without entering credentials</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Inspect the Login page controls without entering credentials.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -540,7 +540,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password input is masked by default while typing</t>
+          <t>Verify password input is masked while entering credentials on the Login page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -556,14 +556,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Click inside the Password field
-Type the password value Carwash#1</t>
+          <t>Open the Login page from the Home page using the person/profile button.
+Click inside the Password field.
+Type the password value Carwash#1 into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered characters and does not display the plain-text password value on screen.</t>
+          <t>The Password field masks the entered characters during input instead of displaying the plain text password value.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful login with approved valid credentials returns the user to authenticated Home state</t>
+          <t>Verify successful login using approved credentials returns the user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -591,15 +591,16 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page
-Enter username krisadmin in the Username field
-Enter password Carwash#1 in the Password field
-Click the Login button</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Enter username value krisadmin in the Username field.
+Enter password value Carwash#1 in the Password field.
+Click the Login button once.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page, removes the guest Home state, replaces the Person/Profile button with the logged-in user identity, and displays authenticated-user features.</t>
+          <t>The application authenticates the user, returns to the Home page in authenticated state, and displays authenticated user identity information together with authenticated-only feature visibility.</t>
         </is>
       </c>
     </row>
@@ -611,12 +612,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify invalid username with valid password does not authenticate the user</t>
+          <t>Verify authenticated Home state is visible after successful login</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -627,15 +628,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter invalid username krisadmin1
-Enter valid password Carwash#1
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Enter approved credentials using username krisadmin and password Carwash#1.
+Submit the login request using the Login button.
+Observe the Home page after authentication completes.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails, an error message is displayed, the application remains on the Login page or unauthenticated state, and authenticated Home controls are not shown.</t>
+          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only feature areas accessible.</t>
         </is>
       </c>
     </row>
@@ -647,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify valid username with invalid password does not authenticate the user</t>
+          <t>Verify invalid username and password combination does not authenticate the user</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -663,15 +664,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter valid username krisadmin
-Enter invalid password Carwash#123
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Enter invalid username value invaliduser in the Username field.
+Enter invalid password value WrongPass#1 in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, visible error feedback is displayed, and the user remains unauthenticated on the Login page.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the user remains unauthenticated, and the application stays on the Login page or otherwise does not enter authenticated Home state.</t>
         </is>
       </c>
     </row>
@@ -683,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify invalid username and invalid password combination is rejected</t>
+          <t>Verify login submission with both Username and Password fields empty displays generic Failed message only</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -699,15 +700,15 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter invalid username invaliduser
-Enter invalid password invalidpass
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Leave the Username field empty.
+Leave the Password field empty.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>The login attempt is rejected with visible authentication error feedback and the application does not transition to authenticated Home state.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -719,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify Login button behavior when Username and Password fields are empty</t>
+          <t>Verify login submission with Username populated and Password empty fails authentication</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -735,15 +736,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Leave the Username field empty
-Leave the Password field empty
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Enter username value krisadmin in the Username field.
+Leave the Password field empty.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Required field validation is displayed for Username and Password, login does not proceed, and the user remains on the Login page.</t>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -755,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify required validation when Username is empty and Password is entered</t>
+          <t>Verify login submission with Password populated and Username empty fails authentication</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -771,15 +772,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Leave the Username field empty
-Enter password Carwash#1
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Leave the Username field empty.
+Enter password value Carwash#1 in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>A Username required validation message is displayed, authentication is blocked, and the Login page remains open.</t>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -791,12 +792,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify required validation when Password is empty and Username is entered</t>
+          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -807,15 +808,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter username krisadmin
-Leave the Password field empty
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Enter username value with leading and trailing spaces around krisadmin into the Username field.
+Enter password value with leading and trailing spaces around Carwash#1 into the Password field.
+Click the Login button and observe the resulting authentication behavior.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>A Password required validation message is displayed, login is not processed, and the user remains on the Login page.</t>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistently applied without application instability or conflicting validation messaging.</t>
         </is>
       </c>
     </row>
@@ -827,7 +828,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify whitespace-only Username and Password values are rejected</t>
+          <t>Verify whitespace-only credential values are rejected with generic Failed message</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -843,15 +844,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter only spaces into the Username field
-Enter only spaces into the Password field
-Click the Login button</t>
+          <t>Open the Login page from the Home page.
+Enter only whitespace characters into the Username field.
+Enter only whitespace characters into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application treats whitespace-only values as invalid input, prevents authentication, and displays validation or authentication error feedback while remaining on the Login page.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -863,12 +864,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify leading and trailing spaces in valid credentials are handled according to business rules</t>
+          <t>Verify Back button returns the user from Login page to unauthenticated Home page</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -879,15 +880,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter username value with leading and trailing spaces around krisadmin
-Enter password value with leading and trailing spaces around Carwash#1
-Click the Login button</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Back button on the Login page.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application consistently handles leading and trailing spaces according to implemented business behavior and the observed authentication result is displayed without causing UI errors or unstable state transitions.</t>
+          <t>The application returns to the Home page in guest unauthenticated state without displaying authenticated user identity or authenticated-only features.</t>
         </is>
       </c>
     </row>
@@ -899,12 +899,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Password field is case-sensitive for authentication</t>
+          <t>Verify Home button returns the user from Login page to unauthenticated Home page</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -915,15 +915,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Enter username krisadmin
-Enter password carwash#1
-Click the Login button</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Home button on the Login page.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Authentication fails for incorrectly cased password input and the Login page remains displayed with authentication error feedback.</t>
+          <t>The application returns to the Home page in guest unauthenticated state without authenticating the user or displaying authenticated-only UI.</t>
         </is>
       </c>
     </row>
@@ -935,12 +934,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user from Login page to Home page</t>
+          <t>Verify all authentication failures display the same generic Failed message</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -951,13 +950,17 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Click the Back button on the Login page</t>
+          <t>Open the Login page from the Home page.
+Attempt login using invalid username and password values and observe the error message.
+Refresh the workflow by reopening the Login page.
+Attempt login with both Username and Password fields blank and observe the error message.
+Refresh the workflow again and reopen the Login page.
+Attempt login with only Username populated and observe the error message.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest state without authenticating the session.</t>
+          <t>Each failed authentication attempt displays the same generic Failed message and does not show separate required-field validation messaging.</t>
         </is>
       </c>
     </row>
@@ -969,12 +972,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user from Login page to Home page</t>
+          <t>Verify extremely long credential values are rejected without breaking Login page behavior</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -985,122 +988,15 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page
-Click the Home button on the Login page</t>
+          <t>Open the Login page from the Home page.
+Enter a very long alphanumeric string exceeding normal username length into the Username field.
+Enter a very long alphanumeric and special character string into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest state and the Login page is closed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-LOGIN16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify authenticated Home state displays logged-in user identity after successful login</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Navigate to the Login page from the Home page
-Enter valid username krisadmin
-Enter valid password Carwash#1
-Click the Login button
-Observe the Home page after authentication completes</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>The Home page displays authenticated-user UI, the guest Person/Profile button is replaced with the logged-in user name, and authenticated-only features become available.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>WT-LOGIN17</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Verify long Username input value is rejected without breaking the Login page</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page
-Enter an excessively long Username value exceeding normal credential length
-Enter password Carwash#1
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>The Login page remains stable, authentication does not succeed with invalid long Username input, and validation or authentication error feedback is displayed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>WT-LOGIN18</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Verify long Password input value is rejected without exposing password text</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page
-Enter username krisadmin
-Enter an excessively long Password value
-Click the Login button</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>The Password field remains masked, authentication fails for invalid long password input, and the Login page remains functional with visible error feedback.</t>
+          <t>The application handles the long credential input without UI corruption or application failure, authentication is rejected, and the generic Failed message is displayed while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 20
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify unauthenticated guest user can open the Login page from the Home page person/profile button</t>
+          <t>Verify guest user can open the Login page from the Home page using the person/profile button</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,15 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open the WashTab application and navigate to http://localhost/washtabui/home.
-Verify the Home page is displayed in guest state without authenticated user identity visible.
+          <t>Launch the WashTab application.
+Navigate to http://localhost/washtabui/home.
+Verify the Home page is displayed in guest state.
 Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the guest Home page to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactive.</t>
+          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactable.</t>
         </is>
       </c>
     </row>
@@ -505,7 +506,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and enabled after opening Login page from Home page</t>
+          <t>Verify Login page controls are visible and enabled after navigation from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -523,12 +524,12 @@
         <is>
           <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Inspect the Login page controls without entering credentials.</t>
+Observe the Username field, Password field, Login button, Back button, and Home button.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Username field, Password field, Login button, Back button, and Home button are visible, enabled, and available for interaction on the Login page.</t>
+          <t>All approved Login page controls are visible, enabled, and available for interaction without UI rendering issues.</t>
         </is>
       </c>
     </row>
@@ -556,14 +557,13 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Click inside the Password field.
-Type the password value Carwash#1 into the Password field.</t>
+          <t>Open the Login page from the Home page person/profile button.
+Enter text into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered characters during input instead of displaying the plain text password value.</t>
+          <t>The Password field masks entered characters during typing and does not display the plain text password value.</t>
         </is>
       </c>
     </row>
@@ -575,7 +575,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful login using approved credentials returns the user to authenticated Home state</t>
+          <t>Verify successful authentication using approved credentials returns user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,14 +593,14 @@
         <is>
           <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Enter username value krisadmin in the Username field.
-Enter password value Carwash#1 in the Password field.
-Click the Login button once.</t>
+Enter Username as krisadmin.
+Enter Password as Carwash#1.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user, returns to the Home page in authenticated state, and displays authenticated user identity information together with authenticated-only feature visibility.</t>
+          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, and authenticated user identity and authenticated-only feature areas become visible.</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify authenticated Home state is visible after successful login</t>
+          <t>Verify authenticated Home page state persists immediately after successful login transition</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -629,14 +629,14 @@
       <c r="F6" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter approved credentials using username krisadmin and password Carwash#1.
-Submit the login request using the Login button.
-Observe the Home page after authentication completes.</t>
+Enter approved credentials with Username krisadmin and Password Carwash#1.
+Click the Login button.
+Observe the Home page after redirection.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only feature areas accessible.</t>
+          <t>The SPA transitions from the Login page to the Home page authenticated state without remaining on the Login page, and authenticated-only UI elements are visible.</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination does not authenticate the user</t>
+          <t>Verify invalid credentials display generic Failed message and keep user unauthenticated</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -665,14 +665,14 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter invalid username value invaliduser in the Username field.
-Enter invalid password value WrongPass#1 in the Password field.
+Enter an invalid Username value.
+Enter an invalid Password value.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, the user remains unauthenticated, and the application stays on the Login page or otherwise does not enter authenticated Home state.</t>
+          <t>Authentication fails, a generic Failed message is displayed, the user remains unauthenticated, and the application does not transition to authenticated Home state.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Verify login submission with both Username and Password fields empty displays generic Failed message only</t>
+          <t>Verify blank Username and blank Password submission displays only generic Failed message</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>Authentication fails, only the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated on the Login page or in guest state.</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify login submission with Username populated and Password empty fails authentication</t>
+          <t>Verify submission with Username populated and Password blank fails authentication</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -737,14 +737,14 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter username value krisadmin in the Username field.
+Enter a Username value.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify login submission with Password populated and Username empty fails authentication</t>
+          <t>Verify submission with Password populated and Username blank fails authentication</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,13 +774,13 @@
         <is>
           <t>Open the Login page from the Home page.
 Leave the Username field empty.
-Enter password value Carwash#1 in the Password field.
+Enter a Password value.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -792,12 +792,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
+          <t>Verify Login page Back button returns user to Home page without authentication</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -808,15 +808,13 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter username value with leading and trailing spaces around krisadmin into the Username field.
-Enter password value with leading and trailing spaces around Carwash#1 into the Password field.
-Click the Login button and observe the resulting authentication behavior.</t>
+          <t>Navigate to the Login page from the Home page.
+Click the Back button.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistently applied without application instability or conflicting validation messaging.</t>
+          <t>The application returns the user to the Home page in guest unauthenticated state and authenticated-only UI is not visible.</t>
         </is>
       </c>
     </row>
@@ -828,12 +826,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify whitespace-only credential values are rejected with generic Failed message</t>
+          <t>Verify Login page Home button returns user to Home page without authentication</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -843,6 +841,77 @@
       </c>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
+Click the Home button.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>The application returns the user to the Home page in guest unauthenticated state and authenticated-only UI is not visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>WT-LOGIN12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Verify leading and trailing whitespace handling for valid credentials</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page.
+Enter Username value with leading and trailing spaces around krisadmin.
+Enter Password value with leading and trailing spaces around Carwash#1.
+Click the Login button.
+Observe the resulting authentication behavior.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistently applied without application instability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WT-LOGIN13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Verify whitespace-only values in Username and Password fields fail authentication with generic Failed message</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
 Enter only whitespace characters into the Username field.
@@ -850,79 +919,9 @@
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>WT-LOGIN12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Verify Back button returns the user from Login page to unauthenticated Home page</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page in guest state.
-Click the person/profile button to open the Login page.
-Click the Back button on the Login page.</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>The application returns to the Home page in guest unauthenticated state without displaying authenticated user identity or authenticated-only features.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>WT-LOGIN13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Verify Home button returns the user from Login page to unauthenticated Home page</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page in guest state.
-Click the person/profile button to open the Login page.
-Click the Home button on the Login page.</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>The application returns to the Home page in guest unauthenticated state without authenticating the user or displaying authenticated-only UI.</t>
         </is>
       </c>
     </row>
@@ -934,12 +933,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify all authentication failures display the same generic Failed message</t>
+          <t>Verify very long credential values do not authenticate and application remains stable</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -951,16 +950,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Attempt login using invalid username and password values and observe the error message.
-Refresh the workflow by reopening the Login page.
-Attempt login with both Username and Password fields blank and observe the error message.
-Refresh the workflow again and reopen the Login page.
-Attempt login with only Username populated and observe the error message.</t>
+Enter an excessively long string into the Username field.
+Enter an excessively long string into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Each failed authentication attempt displays the same generic Failed message and does not show separate required-field validation messaging.</t>
+          <t>Authentication fails safely, the generic Failed message is displayed or the login remains rejected, and the Login page remains stable without broken layout or application crash.</t>
         </is>
       </c>
     </row>
@@ -972,12 +969,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify extremely long credential values are rejected without breaking Login page behavior</t>
+          <t>Verify special characters in Username and Password fields do not bypass authentication</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -989,14 +986,52 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter a very long alphanumeric string exceeding normal username length into the Username field.
-Enter a very long alphanumeric and special character string into the Password field.
+Enter special characters and symbols into the Username field.
+Enter special characters and symbols into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The application handles the long credential input without UI corruption or application failure, authentication is rejected, and the generic Failed message is displayed while the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed, and the user remains unauthenticated without unexpected navigation or script execution behavior.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-LOGIN16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify successful login flow begins only from Home page navigation path</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Navigate to http://localhost/washtabui/home.
+Verify the application is in guest state.
+Click the person/profile button to open the Login page.
+Enter Username as krisadmin.
+Enter Password as Carwash#1.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>The Login workflow is initiated through the Home page person/profile button and successful authentication returns the user to authenticated Home state with authenticated-only UI visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 21
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify guest user can open the Login page from the Home page using the person/profile button</t>
+          <t>Verify unauthenticated guest user can open the Login page from the Home page person/profile button</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,15 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the WashTab application.
-Navigate to http://localhost/washtabui/home.
-Verify the Home page is displayed in guest state.
+          <t>Launch the WashTab application and navigate to http://localhost/washtabui/home.
+Verify the Home page is displayed in guest state without authenticated user identity visible.
 Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactable.</t>
+          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactive.</t>
         </is>
       </c>
     </row>
@@ -506,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and enabled after navigation from Home page</t>
+          <t>Verify Login page controls are visible and interactive after opening Login page from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,85 +521,90 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Navigate to http://localhost/washtabui/home in guest state.
+Click the person/profile button to open the Login page.
+Verify the Username field accepts keyboard focus.
+Verify the Password field accepts keyboard focus.
+Verify the Login button is clickable.
+Verify the Back button is clickable.
+Verify the Home button is clickable.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>All approved Login page controls are visible, enabled, focusable where applicable, and interactive without UI errors or broken SPA state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WT-LOGIN03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Verify password input is masked while typing valid credentials</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page person/profile button.
+Enter krisadmin in the Username field.
+Type Carwash#1 in the Password field.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>The Password field masks the entered password characters during input and the actual password text is not visibly displayed on screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WT-LOGIN04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Verify successful authentication using approved credentials returns user to authenticated Home state</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Observe the Username field, Password field, Login button, Back button, and Home button.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>All approved Login page controls are visible, enabled, and available for interaction without UI rendering issues.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>WT-LOGIN03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Verify password input is masked while entering credentials on the Login page</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page person/profile button.
-Enter text into the Password field.</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>The Password field masks entered characters during typing and does not display the plain text password value.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>WT-LOGIN04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Verify successful authentication using approved credentials returns user to authenticated Home state</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Navigate to the Home page in guest state.
-Click the person/profile button to open the Login page.
-Enter Username as krisadmin.
-Enter Password as Carwash#1.
+Enter krisadmin in the Username field.
+Enter Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, and authenticated user identity and authenticated-only feature areas become visible.</t>
+          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, displays authenticated user identity information, and shows authenticated-only feature areas.</t>
         </is>
       </c>
     </row>
@@ -631,12 +635,12 @@
           <t>Open the Login page from the Home page.
 Enter approved credentials with Username krisadmin and Password Carwash#1.
 Click the Login button.
-Observe the Home page after redirection.</t>
+Observe the Home page after authentication completes.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The SPA transitions from the Login page to the Home page authenticated state without remaining on the Login page, and authenticated-only UI elements are visible.</t>
+          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only features available without showing guest-only unauthenticated state indicators.</t>
         </is>
       </c>
     </row>
@@ -648,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify invalid credentials display generic Failed message and keep user unauthenticated</t>
+          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -664,15 +668,15 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter an invalid Username value.
-Enter an invalid Password value.
+          <t>Open the Login page from the Home page person/profile button.
+Enter invaliduser in the Username field.
+Enter InvalidPass#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Authentication fails, a generic Failed message is displayed, the user remains unauthenticated, and the application does not transition to authenticated Home state.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the application does not transition to authenticated Home state, and the user remains unauthenticated on the Login page or equivalent unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -708,7 +712,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication fails, only the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated on the Login page or in guest state.</t>
+          <t>Authentication fails, only the generic Failed message is displayed, no dedicated required-field validation message is shown, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -720,7 +724,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify submission with Username populated and Password blank fails authentication</t>
+          <t>Verify submission with Username populated and Password blank displays generic Failed message</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -737,14 +741,14 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter a Username value.
+Enter krisadmin in the Username field.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -756,7 +760,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify submission with Password populated and Username blank fails authentication</t>
+          <t>Verify submission with Password populated and Username blank displays generic Failed message</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -774,13 +778,13 @@
         <is>
           <t>Open the Login page from the Home page.
 Leave the Username field empty.
-Enter a Password value.
+Enter Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -792,12 +796,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify Login page Back button returns user to Home page without authentication</t>
+          <t>Verify leading and trailing whitespace handling for approved credentials</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -808,13 +812,16 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Click the Back button.</t>
+          <t>Open the Login page from the Home page.
+Enter space followed by krisadmin followed by trailing spaces in the Username field.
+Enter leading and trailing spaces around Carwash#1 in the Password field.
+Click the Login button.
+Observe the resulting authentication behavior.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest unauthenticated state and authenticated-only UI is not visible.</t>
+          <t>The application handles credential values containing leading or trailing whitespace according to implemented business behavior and the observed result is consistently reflected through either authenticated Home state or the generic Failed message while maintaining correct authentication state.</t>
         </is>
       </c>
     </row>
@@ -826,12 +833,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Login page Home button returns user to Home page without authentication</t>
+          <t>Verify whitespace-only Username and Password values are rejected with generic Failed message</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -842,13 +849,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Click the Home button.</t>
+          <t>Open the Login page from the Home page.
+Enter only space characters in the Username field.
+Enter only space characters in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest unauthenticated state and authenticated-only UI is not visible.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -860,12 +869,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for valid credentials</t>
+          <t>Verify Back button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -876,16 +885,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter Username value with leading and trailing spaces around krisadmin.
-Enter Password value with leading and trailing spaces around Carwash#1.
-Click the Login button.
-Observe the resulting authentication behavior.</t>
+          <t>Navigate to the Login page from the Home page person/profile button.
+Click the Back button on the Login page.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistently applied without application instability.</t>
+          <t>The application returns to the Home page in unauthenticated guest state without displaying authenticated user identity or authenticated-only feature areas.</t>
         </is>
       </c>
     </row>
@@ -897,12 +903,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify whitespace-only values in Username and Password fields fail authentication with generic Failed message</t>
+          <t>Verify Home button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -913,15 +919,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter only whitespace characters into the Username field.
-Enter only whitespace characters into the Password field.
-Click the Login button.</t>
+          <t>Navigate to the Login page from the Home page person/profile button.
+Click the Home button on the Login page.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page in unauthenticated guest state and the user is not authenticated.</t>
         </is>
       </c>
     </row>
@@ -933,12 +937,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify very long credential values do not authenticate and application remains stable</t>
+          <t>Verify invalid password for approved username does not authenticate the user</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -950,14 +954,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter an excessively long string into the Username field.
-Enter an excessively long string into the Password field.
+Enter krisadmin in the Username field.
+Enter WrongPassword#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication fails safely, the generic Failed message is displayed or the login remains rejected, and the Login page remains stable without broken layout or application crash.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the application remains unauthenticated, and authenticated-only Home page features are not displayed.</t>
         </is>
       </c>
     </row>
@@ -969,12 +973,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify special characters in Username and Password fields do not bypass authentication</t>
+          <t>Verify repeated invalid login submissions consistently display the same generic Failed message</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -986,14 +990,13 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter special characters and symbols into the Username field.
-Enter special characters and symbols into the Password field.
-Click the Login button.</t>
+Enter invalid credentials in the Username and Password fields.
+Click the Login button three consecutive times after each failure.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, and the user remains unauthenticated without unexpected navigation or script execution behavior.</t>
+          <t>Each failed authentication attempt displays the same generic Failed message, the user remains unauthenticated, and no additional or inconsistent validation messages are displayed.</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1008,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify successful login flow begins only from Home page navigation path</t>
+          <t>Verify user remains unauthenticated after failed login followed by Home page navigation</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1021,17 +1024,14 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home.
-Verify the application is in guest state.
-Click the person/profile button to open the Login page.
-Enter Username as krisadmin.
-Enter Password as Carwash#1.
-Click the Login button.</t>
+          <t>Open the Login page from the Home page.
+Enter invalid credentials and click the Login button.
+After the Failed message appears, click the Home button.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The Login workflow is initiated through the Home page person/profile button and successful authentication returns the user to authenticated Home state with authenticated-only UI visible.</t>
+          <t>The application returns to the Home page in guest state after the failed login attempt and authenticated user identity information is not displayed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 22
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify unauthenticated guest user can open the Login page from the Home page person/profile button</t>
+          <t>Verify guest user can open the Login page from the Home page using the person/profile button</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the WashTab application and navigate to http://localhost/washtabui/home.
+          <t>Open http://localhost/washtabui/home.
 Verify the Home page is displayed in guest state without authenticated user identity visible.
 Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactive.</t>
+          <t>The application transitions from the guest Home page to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and enabled.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and interactive after opening Login page from Home page</t>
+          <t>Verify Login page controls are visible and interactive after opening from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -521,18 +521,18 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home in guest state.
+          <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Verify the Username field accepts keyboard focus.
-Verify the Password field accepts keyboard focus.
-Verify the Login button is clickable.
-Verify the Back button is clickable.
-Verify the Home button is clickable.</t>
+Click inside the Username field.
+Click inside the Password field.
+Verify the Login button can be clicked.
+Verify the Back button can be clicked.
+Verify the Home button can be clicked.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved Login page controls are visible, enabled, focusable where applicable, and interactive without UI errors or broken SPA state.</t>
+          <t>The Login page opens successfully from the Home page and all approved controls are visible, focusable, and interactive without rendering or navigation issues.</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password input is masked while typing valid credentials</t>
+          <t>Verify password entry is masked during typing on the Login page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -560,14 +560,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page person/profile button.
+          <t>Navigate from the Home page to the Login page using the person/profile button.
 Enter krisadmin in the Username field.
-Type Carwash#1 in the Password field.</t>
+Type Carwash#1 into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered password characters during input and the actual password text is not visibly displayed on screen.</t>
+          <t>The Password field masks the entered password characters during input while retaining the entered value for authentication.</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful authentication using approved credentials returns user to authenticated Home state</t>
+          <t>Verify successful login with approved credentials returns user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -595,8 +595,8 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to the Home page in guest state.
-Click the person/profile button to open the Login page.
+          <t>Open the Home page in guest state.
+Click the person/profile button.
 Enter krisadmin in the Username field.
 Enter Carwash#1 in the Password field.
 Click the Login button.</t>
@@ -604,7 +604,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, displays authenticated user identity information, and shows authenticated-only feature areas.</t>
+          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, displays authenticated user identity information, and displays authenticated-only feature areas.</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify authenticated Home page state persists immediately after successful login transition</t>
+          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -632,15 +632,16 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter approved credentials with Username krisadmin and Password Carwash#1.
-Click the Login button.
-Observe the Home page after authentication completes.</t>
+          <t>Open the Home page in guest state.
+Click the person/profile button.
+Enter invaliduser in the Username field.
+Enter InvalidPassword1! in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only features available without showing guest-only unauthenticated state indicators.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the user remains on the Login page or otherwise unauthenticated, and no authenticated-only Home page features are visible.</t>
         </is>
       </c>
     </row>
@@ -652,7 +653,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
+          <t>Verify blank Username and blank Password submission displays only the generic Failed message</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -668,123 +669,124 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page person/profile button.
-Enter invaliduser in the Username field.
-Enter InvalidPass#1 in the Password field.
-Click the Login button.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed message is displayed, the application does not transition to authenticated Home state, and the user remains unauthenticated on the Login page or equivalent unauthenticated state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WT-LOGIN07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Verify blank Username and blank Password submission displays only generic Failed message</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+          <t>Navigate to the Login page from the Home page.
 Leave the Username field empty.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Authentication fails, only the generic Failed message is displayed, no dedicated required-field validation message is shown, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WT-LOGIN08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Verify submission with Username populated and Password blank displays generic Failed message</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Authentication fails and only the generic Failed message is displayed without any separate required-field validation message, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WT-LOGIN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify login with Username populated and Password empty fails authentication</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
 Enter krisadmin in the Username field.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WT-LOGIN09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Verify submission with Password populated and Username blank displays generic Failed message</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message is shown, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WT-LOGIN08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Verify login with Password populated and Username empty fails authentication</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
 Leave the Username field empty.
 Enter Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message is shown, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WT-LOGIN09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Verify leading and trailing whitespace handling for valid credentials</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
+Enter two leading and trailing spaces around krisadmin in the Username field.
+Enter two leading and trailing spaces around Carwash#1 in the Password field.
+Click the Login button.
+Observe the resulting authentication behavior.</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed authentication result is consistent and stable without application errors.</t>
         </is>
       </c>
     </row>
@@ -796,12 +798,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for approved credentials</t>
+          <t>Verify whitespace-only values in Username and Password fields fail authentication</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -812,16 +814,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter space followed by krisadmin followed by trailing spaces in the Username field.
-Enter leading and trailing spaces around Carwash#1 in the Password field.
-Click the Login button.
-Observe the resulting authentication behavior.</t>
+          <t>Navigate to the Login page from the Home page.
+Enter only spaces into the Username field.
+Enter only spaces into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application handles credential values containing leading or trailing whitespace according to implemented business behavior and the observed result is consistently reflected through either authenticated Home state or the generic Failed message while maintaining correct authentication state.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the user remains unauthenticated, and no dedicated required-field validation message is displayed.</t>
         </is>
       </c>
     </row>
@@ -833,12 +834,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify whitespace-only Username and Password values are rejected with generic Failed message</t>
+          <t>Verify Back button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -849,15 +850,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter only space characters in the Username field.
-Enter only space characters in the Password field.
-Click the Login button.</t>
+          <t>Open the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Back button.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application returns the user to the Home page in guest state without authenticating the user and authenticated-only features remain unavailable.</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user to the Home page without authentication</t>
+          <t>Verify Home button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -885,13 +885,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Click the Back button on the Login page.</t>
+          <t>Open the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Home button.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in unauthenticated guest state without displaying authenticated user identity or authenticated-only feature areas.</t>
+          <t>The application returns the user to the Home page in guest state without authenticating the user and authenticated-only features remain unavailable.</t>
         </is>
       </c>
     </row>
@@ -903,12 +904,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user to the Home page without authentication</t>
+          <t>Verify Login page cannot be considered authenticated after failed login attempt</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -919,13 +920,15 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Click the Home button on the Login page.</t>
+          <t>Navigate to the Login page from the Home page.
+Enter invalid credentials into the Username and Password fields.
+Click the Login button.
+Return to the Home page using the Home button.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in unauthenticated guest state and the user is not authenticated.</t>
+          <t>The generic Failed message is displayed after login submission and the Home page remains in guest state without authenticated user identity or authenticated-only feature visibility.</t>
         </is>
       </c>
     </row>
@@ -937,12 +940,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify invalid password for approved username does not authenticate the user</t>
+          <t>Verify very long Username and Password values do not authenticate and do not break the Login page</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -953,15 +956,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter krisadmin in the Username field.
-Enter WrongPassword#1 in the Password field.
+          <t>Navigate to the Login page from the Home page.
+Enter a very long alphanumeric string exceeding typical username length into the Username field.
+Enter a very long alphanumeric and special character string into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, the application remains unauthenticated, and authenticated-only Home page features are not displayed.</t>
+          <t>Authentication fails safely with the generic Failed message displayed or the values are safely handled without UI corruption, crashes, or unintended authentication.</t>
         </is>
       </c>
     </row>
@@ -973,12 +976,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify repeated invalid login submissions consistently display the same generic Failed message</t>
+          <t>Verify successful authentication updates Home page from guest state to authenticated state</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -989,14 +992,17 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter invalid credentials in the Username and Password fields.
-Click the Login button three consecutive times after each failure.</t>
+          <t>Open the Home page and confirm guest state is visible.
+Click the person/profile button.
+Enter krisadmin in the Username field.
+Enter Carwash#1 in the Password field.
+Click the Login button.
+Observe the Home page after redirection.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Each failed authentication attempt displays the same generic Failed message, the user remains unauthenticated, and no additional or inconsistent validation messages are displayed.</t>
+          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only feature areas available, replacing the previous guest-only state.</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1014,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify user remains unauthenticated after failed login followed by Home page navigation</t>
+          <t>Verify failed authentication does not expose authenticated-only UI elements</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1024,14 +1030,15 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter invalid credentials and click the Login button.
-After the Failed message appears, click the Home button.</t>
+          <t>Navigate to the Login page from the Home page.
+Enter invalid credentials.
+Click the Login button.
+Return to the Home page if still on the Login page.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state after the failed login attempt and authenticated user identity information is not displayed.</t>
+          <t>The user remains unauthenticated after the failed login attempt and authenticated-only Home page features and authenticated identity indicators are not visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 23
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -486,14 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home.
-Verify the Home page is displayed in guest state without authenticated user identity visible.
+          <t>Launch the application and navigate to http://localhost/washtabui/home.
+Verify the Home page is displayed in guest state without authenticated user identity information.
 Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the guest Home page to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and enabled.</t>
+          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactable.</t>
         </is>
       </c>
     </row>
@@ -505,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible and interactive after opening from Home page</t>
+          <t>Verify Login page controls remain visible and interactive after opening from the Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -523,16 +523,13 @@
         <is>
           <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Click inside the Username field.
-Click inside the Password field.
-Verify the Login button can be clicked.
-Verify the Back button can be clicked.
-Verify the Home button can be clicked.</t>
+Inspect the Username field, Password field, Login button, Back button, and Home button.
+Click into the Username and Password fields to confirm they accept input.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The Login page opens successfully from the Home page and all approved controls are visible, focusable, and interactive without rendering or navigation issues.</t>
+          <t>All Login page controls are visible, enabled, and interactive after the Login page opens from the Home page.</t>
         </is>
       </c>
     </row>
@@ -544,7 +541,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password entry is masked during typing on the Login page</t>
+          <t>Verify password input is masked while entering credentials on the Login page</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -560,14 +557,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Navigate from the Home page to the Login page using the person/profile button.
-Enter krisadmin in the Username field.
+          <t>Navigate from the Home page guest state to the Login page using the person/profile button.
+Enter krisadmin into the Username field.
 Type Carwash#1 into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered password characters during input while retaining the entered value for authentication.</t>
+          <t>The Password field masks the entered password characters during input while the Username field remains readable.</t>
         </is>
       </c>
     </row>
@@ -579,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful login with approved credentials returns user to authenticated Home state</t>
+          <t>Verify successful login returns the user to the authenticated Home page state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -595,16 +592,16 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the person/profile button.
-Enter krisadmin in the Username field.
-Enter Carwash#1 in the Password field.
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Enter krisadmin into the Username field.
+Enter Carwash#1 into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, displays authenticated user identity information, and displays authenticated-only feature areas.</t>
+          <t>The application authenticates the user and returns to the Home page in authenticated state with authenticated user identity display and authenticated-only feature area visible.</t>
         </is>
       </c>
     </row>
@@ -616,12 +613,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
+          <t>Verify authenticated Home page state persists immediately after successful login transition</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -632,16 +629,14 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the person/profile button.
-Enter invaliduser in the Username field.
-Enter InvalidPassword1! in the Password field.
-Click the Login button.</t>
+          <t>Open the Login page from the Home page guest state.
+Log in using Username krisadmin and Password Carwash#1.
+Observe the Home page after the authentication redirect completes.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, the user remains on the Login page or otherwise unauthenticated, and no authenticated-only Home page features are visible.</t>
+          <t>The Home page reloads in authenticated state and visibly displays authenticated user identity information together with authenticated-only functionality.</t>
         </is>
       </c>
     </row>
@@ -653,7 +648,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify blank Username and blank Password submission displays only the generic Failed message</t>
+          <t>Verify invalid username and password combination displays the generic Failed message and keeps the user unauthenticated</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -669,87 +664,87 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
+          <t>Navigate from the Home page guest state to the Login page.
+Enter invaliduser into the Username field.
+Enter InvalidPass#1 into the Password field.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, the Login page remains visible or the application remains unauthenticated, and no authenticated Home state is shown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WT-LOGIN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify blank Username and blank Password submission displays only the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page guest state.
 Leave the Username field empty.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Authentication fails and only the generic Failed message is displayed without any separate required-field validation message, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WT-LOGIN07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Verify login with Username populated and Password empty fails authentication</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated on the Login page or in guest state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WT-LOGIN08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Verify login attempt with Username only populated fails with the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
         <is>
           <t>Navigate to the Login page from the Home page.
-Enter krisadmin in the Username field.
+Enter krisadmin into the Username field.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message is shown, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WT-LOGIN08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Verify login with Password populated and Username empty fails authentication</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Navigate to the Login page from the Home page.
-Leave the Username field empty.
-Enter Carwash#1 in the Password field.
-Click the Login button.</t>
-        </is>
-      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message is shown, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -761,12 +756,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for valid credentials</t>
+          <t>Verify login attempt with Password only populated fails with the generic Failed message</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -777,52 +772,51 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
+          <t>Open the Login page from the Home page guest state.
+Leave the Username field empty.
+Enter Carwash#1 into the Password field.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WT-LOGIN10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page through the Home page person/profile button.
 Enter two leading and trailing spaces around krisadmin in the Username field.
 Enter two leading and trailing spaces around Carwash#1 in the Password field.
-Click the Login button.
-Observe the resulting authentication behavior.</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed authentication result is consistent and stable without application errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WT-LOGIN10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Verify whitespace-only values in Username and Password fields fail authentication</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Navigate to the Login page from the Home page.
-Enter only spaces into the Username field.
-Enter only spaces into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, the user remains unauthenticated, and no dedicated required-field validation message is displayed.</t>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the resulting authentication state, redirect behavior, and any Failed message are consistently observable and stable.</t>
         </is>
       </c>
     </row>
@@ -834,12 +828,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user to the Home page without authentication</t>
+          <t>Verify whitespace-only values in Username and Password fields fail authentication with the generic Failed message</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -850,14 +844,15 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the person/profile button to open the Login page.
-Click the Back button.</t>
+          <t>Open the Login page from the Home page.
+Enter only space characters into the Username field.
+Enter only space characters into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest state without authenticating the user and authenticated-only features remain unavailable.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -869,7 +864,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user to the Home page without authentication</t>
+          <t>Verify the Back button returns the user to the Home page without authenticating</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -885,14 +880,13 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
-Click the person/profile button to open the Login page.
-Click the Home button.</t>
+          <t>Navigate to the Login page from the Home page guest state.
+Click the Back button on the Login page.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns the user to the Home page in guest state without authenticating the user and authenticated-only features remain unavailable.</t>
+          <t>The application returns to the Home page in guest state without displaying authenticated user identity information or authenticated-only features.</t>
         </is>
       </c>
     </row>
@@ -904,12 +898,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Login page cannot be considered authenticated after failed login attempt</t>
+          <t>Verify the Home button returns the user to the Home page without authenticating</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -920,15 +914,13 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Enter invalid credentials into the Username and Password fields.
-Click the Login button.
-Return to the Home page using the Home button.</t>
+          <t>Navigate to the Login page from the Home page guest state.
+Click the Home button on the Login page.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The generic Failed message is displayed after login submission and the Home page remains in guest state without authenticated user identity or authenticated-only feature visibility.</t>
+          <t>The application returns to the Home page in guest state and the user remains unauthenticated with authenticated-only UI hidden.</t>
         </is>
       </c>
     </row>
@@ -940,7 +932,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify very long Username and Password values do not authenticate and do not break the Login page</t>
+          <t>Verify very long Username and Password values are handled without breaking the Login page</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -957,14 +949,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Navigate to the Login page from the Home page.
-Enter a very long alphanumeric string exceeding typical username length into the Username field.
-Enter a very long alphanumeric and special character string into the Password field.
+Enter a very long alphanumeric value into the Username field.
+Enter a very long mixed-character value into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Authentication fails safely with the generic Failed message displayed or the values are safely handled without UI corruption, crashes, or unintended authentication.</t>
+          <t>The Login page remains stable, authentication does not succeed with invalid long credentials, and the generic Failed message is displayed while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -976,7 +968,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify successful authentication updates Home page from guest state to authenticated state</t>
+          <t>Verify Login page navigation sequence preserves Home-to-Login-to-Home SPA behavior</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -992,53 +984,15 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open the Home page and confirm guest state is visible.
-Click the person/profile button.
-Enter krisadmin in the Username field.
-Enter Carwash#1 in the Password field.
-Click the Login button.
-Observe the Home page after redirection.</t>
+          <t>Navigate to http://localhost/washtabui/home and verify guest state.
+Click the person/profile button to open the Login page.
+Log in using Username krisadmin and Password Carwash#1.
+Observe the destination page after authentication.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The Home page reloads in authenticated state with authenticated user identity visible and authenticated-only feature areas available, replacing the previous guest-only state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>WT-LOGIN16</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Verify failed authentication does not expose authenticated-only UI elements</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Navigate to the Login page from the Home page.
-Enter invalid credentials.
-Click the Login button.
-Return to the Home page if still on the Login page.</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>The user remains unauthenticated after the failed login attempt and authenticated-only Home page features and authenticated identity indicators are not visible.</t>
+          <t>The workflow follows the approved SPA navigation sequence from Home page guest state to Login page and back to the Home page in authenticated state without requiring direct Login page URL access.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 25
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -487,13 +487,13 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Open http://localhost/washtabui/home.
-Verify the Home page is displayed in guest state and the user is unauthenticated.
+Verify the application is displaying the Home page in guest state.
 Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page guest state to the Login page while remaining unauthenticated and the Login view is displayed successfully.</t>
+          <t>The application transitions from the Home page guest state to the Login page with Username, Password, Login, Back, and Home controls visible while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -521,16 +521,18 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
+          <t>Open http://localhost/washtabui/home.
 Click the person/profile button to open the Login page.
-Observe the Username field, Password field, Login button, Back button, and Home button.
-Click into the Username and Password fields and verify text entry is possible.
-Verify the Login, Back, and Home buttons are clickable.</t>
+Verify the Username field is visible and accepts input.
+Verify the Password field is visible and accepts input.
+Verify the Login button is visible and clickable.
+Verify the Back button is visible and clickable.
+Verify the Home button is visible and clickable.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Username, Password, Login, Back, and Home controls are visible, enabled, and interactive on the Login page.</t>
+          <t>All approved Login page controls are visible, enabled, interactive, and ready for user interaction on the Login page.</t>
         </is>
       </c>
     </row>
@@ -542,7 +544,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify password field masks entered characters during credential entry</t>
+          <t>Verify Password field masks entered characters during credential entry</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -558,14 +560,14 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page person/profile button.
-Enter text into the Username field.
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter krisadmin into the Username field.
 Type Carwash#1 into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks the entered password characters instead of displaying the plain text value.</t>
+          <t>The Password field displays masked characters instead of the actual password value while retaining the entered password for submission.</t>
         </is>
       </c>
     </row>
@@ -577,7 +579,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful authentication with approved credentials returns the user to authenticated Home state</t>
+          <t>Verify successful authentication using approved credentials returns the user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -593,16 +595,16 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open the Home page in guest state.
+          <t>Open http://localhost/washtabui/home and verify the user is unauthenticated.
 Click the person/profile button to open the Login page.
-Enter username krisadmin into the Username field.
-Enter password Carwash#1 into the Password field.
+Enter krisadmin into the Username field.
+Enter Carwash#1 into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, and authenticated user identity and authenticated-only feature areas are visible.</t>
+          <t>The application authenticates the user and returns to the Home page in authenticated state with authenticated user identity information and authenticated-only feature area visible.</t>
         </is>
       </c>
     </row>
@@ -614,12 +616,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify authenticated Home state is visible after successful login</t>
+          <t>Verify invalid username and password combination displays the generic Failed message and keeps the user unauthenticated</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -630,15 +632,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter approved credentials using username krisadmin and password Carwash#1.
-Click the Login button.
-Observe the returned Home page state after authentication completes.</t>
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter invaliduser into the Username field.
+Enter InvalidPassword#1 into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home page reloads in authenticated state with authenticated user identity displayed and authenticated-only features visible.</t>
+          <t>The generic Failed authentication message is displayed, the user remains unauthenticated, and the application stays on the Login page or otherwise does not enter authenticated Home state.</t>
         </is>
       </c>
     </row>
@@ -650,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
+          <t>Verify submitting the Login form with both Username and Password empty displays only the generic Failed message</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -666,123 +668,123 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter invalidUser into the Username field.
-Enter InvalidPassword#1 into the Password field.
-Click the Login button.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed message is displayed, the user remains unauthenticated, and the application stays on the Login page or otherwise does not enter authenticated Home state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WT-LOGIN07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Verify blank Username and blank Password submission displays only generic Failed message</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+          <t>Open the Login page from the Home page using the person/profile button.
 Leave the Username field empty.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Authentication fails and only the generic Failed message is displayed without separate required-field validation messaging, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WT-LOGIN08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Verify login attempt with only Username populated fails and keeps user unauthenticated</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>The application displays only the generic Failed authentication message, no dedicated required-field validation message is shown, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WT-LOGIN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify submitting only Username without Password fails authentication and preserves unauthenticated state</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page using the person/profile button.
 Enter krisadmin into the Username field.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WT-LOGIN09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Verify login attempt with only Password populated fails and keeps user unauthenticated</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>The generic Failed authentication message is displayed without separate required-field validation messaging and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WT-LOGIN08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Verify submitting only Password without Username fails authentication and preserves unauthenticated state</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page using the person/profile button.
 Leave the Username field empty.
 Enter Carwash#1 into the Password field.
 Click the Login button.</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>The generic Failed authentication message is displayed without separate required-field validation messaging and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WT-LOGIN09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter two leading spaces and two trailing spaces around krisadmin in the Username field.
+Enter two leading spaces and two trailing spaces around Carwash#1 in the Password field.
+Click the Login button.</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application handles credential values containing leading and trailing whitespace according to implemented business behavior and the resulting authenticated or failed state is displayed consistently with observable UI feedback.</t>
         </is>
       </c>
     </row>
@@ -794,12 +796,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for valid credentials</t>
+          <t>Verify whitespace-only Username and Password submission displays the generic Failed message</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -810,16 +812,15 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter value with leading and trailing spaces around krisadmin into the Username field.
-Enter value with leading and trailing spaces around Carwash#1 into the Password field.
-Click the Login button.
-Observe the authentication result and returned application state.</t>
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter only whitespace characters into the Username field.
+Enter only whitespace characters into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed authentication outcome is consistent, with either successful authenticated Home navigation or the generic Failed message while remaining unauthenticated.</t>
+          <t>The generic Failed authentication message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -831,12 +832,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify whitespace-only values in Username and Password fields fail authentication</t>
+          <t>Verify the Back button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -847,15 +848,13 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter only spaces into the Username field.
-Enter only spaces into the Password field.
-Click the Login button.</t>
+          <t>Open the Login page from the Home page using the person/profile button.
+Click the Back button.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page in guest state without displaying authenticated user identity information or authenticated-only functionality.</t>
         </is>
       </c>
     </row>
@@ -867,7 +866,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user to Home page without authentication</t>
+          <t>Verify the Home button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -884,12 +883,12 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page using the person/profile button.
-Click the Back button on the Login page.</t>
+Click the Home button.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state without authenticating the user and authenticated-only UI is not visible.</t>
+          <t>The application returns to the Home page in guest state without authenticating the user and guest-state behavior remains visible.</t>
         </is>
       </c>
     </row>
@@ -901,12 +900,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user to Home page without authentication</t>
+          <t>Verify very long Username and Password values are rejected without authenticating the user</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -918,12 +917,14 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page using the person/profile button.
-Click the Home button on the Login page.</t>
+Enter a very long alphanumeric string exceeding normal credential length into the Username field.
+Enter a very long mixed-character password value into the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state without authenticating the user and authenticated-only UI is not visible.</t>
+          <t>The application rejects the authentication attempt, displays the generic Failed message, remains stable, and keeps the user unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -935,7 +936,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify failed authentication keeps Login page controls accessible for another attempt</t>
+          <t>Verify user remains unauthenticated after failed login followed by Home page return navigation</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -951,14 +952,54 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Submit invalid credentials using the Login button.
-After the generic Failed message appears, attempt to interact with the Username field, Password field, and Login button again.</t>
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter invaliduser into the Username field.
+Enter WrongPassword#1 into the Password field.
+Click the Login button.
+Click the Home button.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>After failed authentication, the Login page remains accessible, the Username and Password fields remain interactive, the Login button remains usable, and the user stays unauthenticated.</t>
+          <t>The user returns to the Home page in guest state after the failed login attempt and authenticated user identity or authenticated-only feature areas are not visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WT-LOGIN15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Verify navigation sequence preserves Home-to-Login-to-Home authenticated transition behavior</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Open http://localhost/washtabui/home.
+Verify the Home page is in guest state.
+Click the person/profile button to open the Login page.
+Enter krisadmin into the Username field.
+Enter Carwash#1 into the Password field.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>The workflow follows the approved Home-to-Login-to-Home navigation sequence and finishes on the authenticated Home page with authenticated identity and authenticated-only features visible.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 26
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Login page opens from Home page guest state using the person/profile button</t>
+          <t>Verify Home guest state opens Login page through the person/profile button navigation flow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,14 +486,15 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home.
-Verify the application is displaying the Home page in guest state.
-Click the person/profile button on the Home page.</t>
+          <t>Launch the application and navigate to http://localhost/washtabui/home.
+Verify the application is in Home guest state and the user is unauthenticated.
+Click the person/profile button on the Home page.
+Observe the Login page transition and available controls.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the Home page guest state to the Login page with Username, Password, Login, Back, and Home controls visible while the user remains unauthenticated.</t>
+          <t>The application transitions from the Home guest state to the Login page through the person/profile button flow and the Username, Password, Login, Back, and Home controls are visible and interactive while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -521,18 +522,16 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home.
+          <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Verify the Username field is visible and accepts input.
-Verify the Password field is visible and accepts input.
-Verify the Login button is visible and clickable.
-Verify the Back button is visible and clickable.
-Verify the Home button is visible and clickable.</t>
+Click inside the Username field.
+Click inside the Password field.
+Hover over and click the Login button, Back button, and Home button without submitting credentials.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>All approved Login page controls are visible, enabled, interactive, and ready for user interaction on the Login page.</t>
+          <t>The Username field, Password field, Login button, Back button, and Home button are visible, enabled, clickable, and accept user interaction without displaying authentication errors.</t>
         </is>
       </c>
     </row>
@@ -544,7 +543,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Verify Password field masks entered characters during credential entry</t>
+          <t>Verify password input remains masked during credential entry</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -560,14 +559,15 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
+          <t>Navigate to the Login page from the Home page person/profile button.
 Enter krisadmin into the Username field.
-Type Carwash#1 into the Password field.</t>
+Type Carwash#1 into the Password field.
+Observe the Password field while entering characters.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field displays masked characters instead of the actual password value while retaining the entered password for submission.</t>
+          <t>The Password field masks all entered password characters during input entry and does not display the plain text password value.</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful authentication using approved credentials returns the user to authenticated Home state</t>
+          <t>Verify successful login with approved credentials returns the user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -595,16 +595,16 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home and verify the user is unauthenticated.
+          <t>Navigate to http://localhost/washtabui/home and confirm guest state.
 Click the person/profile button to open the Login page.
-Enter krisadmin into the Username field.
-Enter Carwash#1 into the Password field.
+Enter Username value krisadmin.
+Enter Password value Carwash#1.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user and returns to the Home page in authenticated state with authenticated user identity information and authenticated-only feature area visible.</t>
+          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, and authenticated-only UI with authenticated user identity information becomes visible.</t>
         </is>
       </c>
     </row>
@@ -616,12 +616,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination displays the generic Failed message and keeps the user unauthenticated</t>
+          <t>Verify authenticated Home page state persists immediately after successful login transition</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -632,15 +632,15 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Enter invaliduser into the Username field.
-Enter InvalidPassword#1 into the Password field.
-Click the Login button.</t>
+          <t>Open the Login page from the Home page.
+Enter valid credentials using krisadmin and Carwash#1.
+Click the Login button.
+Observe the Home page after the authentication redirect completes.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The generic Failed authentication message is displayed, the user remains unauthenticated, and the application stays on the Login page or otherwise does not enter authenticated Home state.</t>
+          <t>The Home page reloads in authenticated state and displays authenticated user identity information and authenticated-only features instead of guest-only unauthenticated state behavior.</t>
         </is>
       </c>
     </row>
@@ -652,7 +652,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify submitting the Login form with both Username and Password empty displays only the generic Failed message</t>
+          <t>Verify invalid username and password combination displays the generic Failed message and blocks authentication</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -668,123 +668,123 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
+          <t>Navigate to the Login page from the Home page person/profile button.
+Enter invalid Username value invaliduser.
+Enter invalid Password value InvalidPass#1.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed authentication message is displayed, the user remains unauthenticated, and the application does not transition to authenticated Home state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WT-LOGIN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify blank Username and blank Password submission displays only the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page.
 Leave the Username field empty.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>The application displays only the generic Failed authentication message, no dedicated required-field validation message is shown, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WT-LOGIN07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Verify submitting only Username without Password fails authentication and preserves unauthenticated state</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated on the Login page or in guest state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>WT-LOGIN08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Verify submission with only Username populated fails authentication with the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page using the person/profile button.
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
 Enter krisadmin into the Username field.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>The generic Failed authentication message is displayed without separate required-field validation messaging and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>WT-LOGIN08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Verify submitting only Password without Username fails authentication and preserves unauthenticated state</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WT-LOGIN09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Verify submission with only Password populated fails authentication with the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page using the person/profile button.
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
 Leave the Username field empty.
 Enter Carwash#1 into the Password field.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>The generic Failed authentication message is displayed without separate required-field validation messaging and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WT-LOGIN09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Edge</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Enter two leading spaces and two trailing spaces around krisadmin in the Username field.
-Enter two leading spaces and two trailing spaces around Carwash#1 in the Password field.
-Click the Login button.</t>
-        </is>
-      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>The application handles credential values containing leading and trailing whitespace according to implemented business behavior and the resulting authenticated or failed state is displayed consistently with observable UI feedback.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -796,12 +796,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify whitespace-only Username and Password submission displays the generic Failed message</t>
+          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -812,49 +812,52 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
+          <t>Open the Login page from the Home page.
+Enter Username value with leading and trailing spaces around krisadmin.
+Enter Password value with leading and trailing spaces around Carwash#1.
+Click the Login button.
+Observe the resulting authentication behavior.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistent, stable, and clearly indicates either authenticated Home state or generic Failed authentication behavior without unexpected validation messages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>WT-LOGIN11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Verify whitespace-only Username and Password values fail authentication using the generic Failed message</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
 Enter only whitespace characters into the Username field.
 Enter only whitespace characters into the Password field.
 Click the Login button.</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>The generic Failed authentication message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>WT-LOGIN11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Verify the Back button returns the user to the Home page without authentication</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Click the Back button.</t>
-        </is>
-      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state without displaying authenticated user identity information or authenticated-only functionality.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -866,7 +869,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify the Home button returns the user to the Home page without authentication</t>
+          <t>Verify Back button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -882,13 +885,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Click the Home button.</t>
+          <t>Navigate to the Login page from the Home page person/profile button.
+Click the Back button on the Login page.
+Observe the resulting page state.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest state without authenticating the user and guest-state behavior remains visible.</t>
+          <t>The application returns to the Home page in guest unauthenticated state without displaying authenticated user identity or authenticated-only features.</t>
         </is>
       </c>
     </row>
@@ -900,12 +904,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify very long Username and Password values are rejected without authenticating the user</t>
+          <t>Verify Home button returns the user to the Home page without authentication</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -916,15 +920,14 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Enter a very long alphanumeric string exceeding normal credential length into the Username field.
-Enter a very long mixed-character password value into the Password field.
-Click the Login button.</t>
+          <t>Navigate to the Login page from the Home page person/profile button.
+Click the Home button on the Login page.
+Observe the resulting page state.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application rejects the authentication attempt, displays the generic Failed message, remains stable, and keeps the user unauthenticated.</t>
+          <t>The application returns to the Home page in guest unauthenticated state without authenticating the user or exposing authenticated-only features.</t>
         </is>
       </c>
     </row>
@@ -936,7 +939,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify user remains unauthenticated after failed login followed by Home page return navigation</t>
+          <t>Verify failed authentication keeps the application on Login flow without authenticated transition</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -952,16 +955,15 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page using the person/profile button.
-Enter invaliduser into the Username field.
-Enter WrongPassword#1 into the Password field.
+          <t>Open the Login page from the Home page.
+Enter invalid Username and Password values.
 Click the Login button.
-Click the Home button.</t>
+Observe the application state after the failure message appears.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The user returns to the Home page in guest state after the failed login attempt and authenticated user identity or authenticated-only feature areas are not visible.</t>
+          <t>The application does not transition to authenticated Home state, the generic Failed message remains visible, and the user stays unauthenticated on the Login page or equivalent unauthenticated state.</t>
         </is>
       </c>
     </row>
@@ -973,12 +975,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify navigation sequence preserves Home-to-Login-to-Home authenticated transition behavior</t>
+          <t>Verify special character input in Username and Password fields does not bypass authentication validation</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -989,17 +991,51 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Open http://localhost/washtabui/home.
-Verify the Home page is in guest state.
-Click the person/profile button to open the Login page.
-Enter krisadmin into the Username field.
-Enter Carwash#1 into the Password field.
+          <t>Open the Login page from the Home page.
+Enter special-character-heavy text into the Username field.
+Enter special-character-heavy text into the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>The workflow follows the approved Home-to-Login-to-Home navigation sequence and finishes on the authenticated Home page with authenticated identity and authenticated-only features visible.</t>
+          <t>Authentication fails safely, the generic Failed message is displayed, the application remains stable, and the user stays unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WT-LOGIN16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Verify very long Username and Password values do not authenticate the user and do not break Login page behavior</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Navigate to the Login page from the Home page.
+Enter a very long Username value exceeding normal credential length.
+Enter a very long Password value exceeding normal credential length.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Authentication fails with the generic Failed message or equivalent rejected authentication behavior, the Login page remains responsive, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Multi Page Workflow Commit Part 27
</commit_message>
<xml_diff>
--- a/manual_tests/login/login_approved_manual_tests.xlsx
+++ b/manual_tests/login/login_approved_manual_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -470,7 +470,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Verify Home guest state opens Login page through the person/profile button navigation flow</t>
+          <t>Verify Login page opens from Home page using the person/profile button while user is in guest state</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -486,15 +486,14 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Launch the application and navigate to http://localhost/washtabui/home.
-Verify the application is in Home guest state and the user is unauthenticated.
-Click the person/profile button on the Home page.
-Observe the Login page transition and available controls.</t>
+          <t>Navigate to http://localhost/washtabui/home.
+Verify the Home page is displayed in guest state without authenticated user identity information.
+Click the person/profile button on the Home page.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>The application transitions from the Home guest state to the Login page through the person/profile button flow and the Username, Password, Login, Back, and Home controls are visible and interactive while the user remains unauthenticated.</t>
+          <t>The application transitions from the Home page guest state to the Login page and the Username field, Password field, Login button, Back button, and Home button are visible and interactive while the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -506,7 +505,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Verify Login page controls are visible, enabled, and interactive after opening from Home page</t>
+          <t>Verify Login page controls are visible and enabled after opening Login page from Home page</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -522,52 +521,50 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
+          <t>Navigate to http://localhost/washtabui/home.
+Click the person/profile button to open the Login page.
+Observe the Login page controls without entering credentials.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>The Username field, Password field, Login button, Back button, and Home button are visible, enabled, and available for interaction on the Login page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>WT-LOGIN03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Verify password input is masked while entering password characters</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Navigate to the Home page in guest state.
 Click the person/profile button to open the Login page.
-Click inside the Username field.
-Click inside the Password field.
-Hover over and click the Login button, Back button, and Home button without submitting credentials.</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>The Username field, Password field, Login button, Back button, and Home button are visible, enabled, clickable, and accept user interaction without displaying authentication errors.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>WT-LOGIN03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Verify password input remains masked during credential entry</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Enter krisadmin into the Username field.
-Type Carwash#1 into the Password field.
-Observe the Password field while entering characters.</t>
+Enter krisadmin in the Username field.
+Type Carwash#1 into the Password field.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>The Password field masks all entered password characters during input entry and does not display the plain text password value.</t>
+          <t>The Password field masks the entered password characters during input and does not display the plain text password value visibly on screen.</t>
         </is>
       </c>
     </row>
@@ -579,7 +576,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Verify successful login with approved credentials returns the user to authenticated Home state</t>
+          <t>Verify successful login using approved credentials returns user to authenticated Home state</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -595,16 +592,17 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Navigate to http://localhost/washtabui/home and confirm guest state.
-Click the person/profile button to open the Login page.
-Enter Username value krisadmin.
-Enter Password value Carwash#1.
+          <t>Navigate to http://localhost/washtabui/home.
+Verify the application is in Home guest state.
+Click the person/profile button.
+Enter krisadmin in the Username field.
+Enter Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>The application authenticates the user successfully, returns to the Home page in authenticated state, and authenticated-only UI with authenticated user identity information becomes visible.</t>
+          <t>The application authenticates the user successfully and returns to the Home page in authenticated state with authenticated user identity display and authenticated-only feature area visible.</t>
         </is>
       </c>
     </row>
@@ -616,12 +614,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Verify authenticated Home page state persists immediately after successful login transition</t>
+          <t>Verify invalid username and password combination displays generic Failed message and keeps user unauthenticated</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -632,15 +630,16 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Open the Login page from the Home page.
-Enter valid credentials using krisadmin and Carwash#1.
-Click the Login button.
-Observe the Home page after the authentication redirect completes.</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button.
+Enter invaliduser in the Username field.
+Enter Invalid#123 in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>The Home page reloads in authenticated state and displays authenticated user identity information and authenticated-only features instead of guest-only unauthenticated state behavior.</t>
+          <t>Authentication fails, the generic Failed message is displayed, the application does not transition to authenticated Home state, and the user remains unauthenticated on the Login page or Home guest state.</t>
         </is>
       </c>
     </row>
@@ -652,7 +651,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Verify invalid username and password combination displays the generic Failed message and blocks authentication</t>
+          <t>Verify login submission with both Username and Password fields empty displays only the generic Failed message</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -668,51 +667,52 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Enter invalid Username value invaliduser.
-Enter invalid Password value InvalidPass#1.
-Click the Login button.</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Authentication fails, the generic Failed authentication message is displayed, the user remains unauthenticated, and the application does not transition to authenticated Home state.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>WT-LOGIN07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Verify blank Username and blank Password submission displays only the generic Failed message</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Open the Login page from the Home page.
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button.
 Leave the Username field empty.
 Leave the Password field empty.
 Click the Login button.</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>WT-LOGIN07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Verify login submission with Username populated and Password empty displays generic Failed message</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page using the person/profile button.
+Enter krisadmin in the Username field.
+Leave the Password field empty.
+Click the Login button.</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated on the Login page or in guest state.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Verify submission with only Username populated fails authentication with the generic Failed message</t>
+          <t>Verify login submission with Password populated and Username empty displays generic Failed message</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -740,15 +740,15 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Enter krisadmin into the Username field.
-Leave the Password field empty.
+          <t>Open the Login page from the Home page using the person/profile button.
+Leave the Username field empty.
+Enter Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -760,12 +760,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Verify submission with only Password populated fails authentication with the generic Failed message</t>
+          <t>Verify login attempt with leading and trailing spaces around valid credentials follows implemented whitespace handling behavior</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -776,15 +776,15 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Leave the Username field empty.
-Enter Carwash#1 into the Password field.
+          <t>Open the Login page from the Home page.
+Enter two leading spaces and two trailing spaces around krisadmin in the Username field.
+Enter two leading spaces and two trailing spaces around Carwash#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application handles leading and trailing whitespace according to implemented business behavior and the resulting authentication state and visible response are consistent and observable without application instability.</t>
         </is>
       </c>
     </row>
@@ -796,12 +796,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Verify leading and trailing whitespace handling for Username and Password values</t>
+          <t>Verify whitespace-only values in Username and Password fields display generic Failed message</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -813,15 +813,14 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter Username value with leading and trailing spaces around krisadmin.
-Enter Password value with leading and trailing spaces around Carwash#1.
-Click the Login button.
-Observe the resulting authentication behavior.</t>
+Enter only whitespace characters in the Username field.
+Enter only whitespace characters in the Password field.
+Click the Login button.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>The application handles leading and trailing whitespace according to implemented business behavior and the observed result is consistent, stable, and clearly indicates either authenticated Home state or generic Failed authentication behavior without unexpected validation messages.</t>
+          <t>Authentication fails, the generic Failed message is displayed, no separate required-field validation appears, and the user remains unauthenticated.</t>
         </is>
       </c>
     </row>
@@ -833,12 +832,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Verify whitespace-only Username and Password values fail authentication using the generic Failed message</t>
+          <t>Verify Back button returns the user to Home page without authentication</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -849,15 +848,14 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Enter only whitespace characters into the Username field.
-Enter only whitespace characters into the Password field.
-Click the Login button.</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Back button on the Login page.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Authentication fails, the generic Failed message is displayed, no dedicated required-field validation message appears, and the user remains unauthenticated.</t>
+          <t>The application returns to the Home page in guest state and authenticated user identity information is not visible.</t>
         </is>
       </c>
     </row>
@@ -869,7 +867,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Verify Back button returns the user to the Home page without authentication</t>
+          <t>Verify Home button returns the user to Home page without authentication</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -885,14 +883,14 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Click the Back button on the Login page.
-Observe the resulting page state.</t>
+          <t>Navigate to the Home page in guest state.
+Click the person/profile button to open the Login page.
+Click the Home button on the Login page.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest unauthenticated state without displaying authenticated user identity or authenticated-only features.</t>
+          <t>The application returns to the Home page in guest state and authenticated-only feature areas are not visible.</t>
         </is>
       </c>
     </row>
@@ -904,12 +902,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Verify Home button returns the user to the Home page without authentication</t>
+          <t>Verify generic Failed message remains consistent across multiple invalid authentication attempts</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -920,14 +918,16 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page person/profile button.
-Click the Home button on the Login page.
-Observe the resulting page state.</t>
+          <t>Open the Login page from the Home page.
+Submit invalid credentials using invaliduser and Invalid#123.
+Observe the displayed authentication failure message.
+Clear the fields and submit a blank Username and blank Password login request.
+Observe the displayed authentication failure message again.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>The application returns to the Home page in guest unauthenticated state without authenticating the user or exposing authenticated-only features.</t>
+          <t>Each authentication failure displays the same generic Failed message without separate validation wording and the user remains unauthenticated after each attempt.</t>
         </is>
       </c>
     </row>
@@ -939,12 +939,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verify failed authentication keeps the application on Login flow without authenticated transition</t>
+          <t>Verify successful login state displays authenticated-only UI after returning to Home page</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -956,14 +956,14 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter invalid Username and Password values.
+Enter approved credentials krisadmin and Carwash#1.
 Click the Login button.
-Observe the application state after the failure message appears.</t>
+Observe the Home page after authentication completes.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>The application does not transition to authenticated Home state, the generic Failed message remains visible, and the user stays unauthenticated on the Login page or equivalent unauthenticated state.</t>
+          <t>The Home page reloads in authenticated state with authenticated user identity display and authenticated-only feature area visible to the signed-in user.</t>
         </is>
       </c>
     </row>
@@ -975,12 +975,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Verify special character input in Username and Password fields does not bypass authentication validation</t>
+          <t>Verify credential fields accept special characters in password input without breaking masking behavior</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Edge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -992,14 +992,13 @@
       <c r="F16" t="inlineStr">
         <is>
           <t>Open the Login page from the Home page.
-Enter special-character-heavy text into the Username field.
-Enter special-character-heavy text into the Password field.
-Click the Login button.</t>
+Enter krisadmin in the Username field.
+Enter Carwash#1 in the Password field and observe the field while typing.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Authentication fails safely, the generic Failed message is displayed, the application remains stable, and the user stays unauthenticated.</t>
+          <t>The Password field accepts special characters such as # while maintaining masked password display behavior.</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1010,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Verify very long Username and Password values do not authenticate the user and do not break Login page behavior</t>
+          <t>Verify invalid credentials with correct username and incorrect password do not authenticate the user</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Edge</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1027,15 +1026,51 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Navigate to the Login page from the Home page.
-Enter a very long Username value exceeding normal credential length.
-Enter a very long Password value exceeding normal credential length.
+          <t>Open the Login page from the Home page.
+Enter krisadmin in the Username field.
+Enter WrongPassword#1 in the Password field.
 Click the Login button.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Authentication fails with the generic Failed message or equivalent rejected authentication behavior, the Login page remains responsive, and the user remains unauthenticated.</t>
+          <t>Authentication fails, the generic Failed message is displayed, and the user remains unauthenticated without access to authenticated Home features.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WT-LOGIN17</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Verify invalid credentials with incorrect username and correct password do not authenticate the user</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Open the Login page from the Home page.
+Enter wronguser in the Username field.
+Enter Carwash#1 in the Password field.
+Click the Login button.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Authentication fails, the generic Failed message is displayed, and the application does not transition to authenticated Home state.</t>
         </is>
       </c>
     </row>

</xml_diff>